<commit_message>
Add per-touch Contribution Type and Handoff Quality scoring
Adds two new Case Tracker columns (Contribution Type: Resolver/Progress
Builder/Maintainer/Breaker, and Handoff Quality 0-5) with dropdowns,
conditional formatting, and the worked Stell journey tagged. Adds a
methodology section to the Multi-Touch Guide and a live per-touch
breakdown table to the Team Scoring sheet to inform the Continuity score.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form.xlsx
+++ b/QA Scoring Form.xlsx
@@ -211,7 +211,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -349,11 +349,55 @@
         <color rgb="001F3864"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="001F3864"/>
+      </right>
+      <top style="thick">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="001F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="001F3864"/>
+      </right>
+      <top style="thick">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="001F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -715,11 +759,31 @@
     <xf numFmtId="0" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
     <dxf>
       <font>
         <b val="1"/>
@@ -912,6 +976,17 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001F3864"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9E1F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1731,7 +1806,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="104" t="inlineStr">
         <is>
           <t>SUPPORT QUALITY ASSURANCE — SCORING FORM</t>
         </is>
@@ -1753,7 +1828,7 @@
       <c r="F2" s="68" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="71" t="inlineStr">
+      <c r="B4" s="116" t="inlineStr">
         <is>
           <t>1 · CASE INFORMATION</t>
         </is>
@@ -1917,7 +1992,7 @@
       <c r="F16" s="68" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="71" t="inlineStr">
+      <c r="B17" s="116" t="inlineStr">
         <is>
           <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
@@ -2067,7 +2142,7 @@
       <c r="F28" s="69" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="71" t="inlineStr">
+      <c r="B30" s="116" t="inlineStr">
         <is>
           <t>2. TECHNICAL ACCURACY</t>
         </is>
@@ -2239,7 +2314,7 @@
       <c r="F43" s="69" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="B45" s="71" t="inlineStr">
+      <c r="B45" s="116" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
@@ -2422,7 +2497,7 @@
       <c r="F59" s="69" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="B61" s="71" t="inlineStr">
+      <c r="B61" s="116" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
@@ -2605,7 +2680,7 @@
       <c r="F75" s="69" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="B77" s="71" t="inlineStr">
+      <c r="B77" s="116" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
@@ -2755,7 +2830,7 @@
       <c r="F88" s="69" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="B90" s="71" t="inlineStr">
+      <c r="B90" s="116" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
@@ -2916,7 +2991,7 @@
       <c r="F102" s="69" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="B104" s="71" t="inlineStr">
+      <c r="B104" s="116" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
@@ -3099,27 +3174,27 @@
       <c r="F119" s="68" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="75" t="inlineStr">
+      <c r="B120" s="118" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C120" s="75" t="inlineStr">
+      <c r="C120" s="118" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D120" s="75" t="inlineStr">
+      <c r="D120" s="118" t="inlineStr">
         <is>
           <t>Score (0-5)</t>
         </is>
       </c>
-      <c r="E120" s="75" t="inlineStr">
+      <c r="E120" s="118" t="inlineStr">
         <is>
           <t>Weighted</t>
         </is>
       </c>
-      <c r="F120" s="75" t="inlineStr">
+      <c r="F120" s="118" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
@@ -3300,7 +3375,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="71" t="inlineStr">
+      <c r="B130" s="116" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
@@ -3344,7 +3419,7 @@
       <c r="F133" s="69" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="71" t="inlineStr">
+      <c r="B135" s="116" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
@@ -3392,7 +3467,7 @@
       <c r="F137" s="69" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="39" t="inlineStr">
+      <c r="B139" s="121" t="inlineStr">
         <is>
           <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
         </is>
@@ -3403,17 +3478,17 @@
       <c r="F139" s="68" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="71" t="inlineStr">
+      <c r="B140" s="116" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="C140" s="75" t="inlineStr">
+      <c r="C140" s="118" t="inlineStr">
         <is>
           <t>Present?</t>
         </is>
       </c>
-      <c r="D140" s="71" t="inlineStr">
+      <c r="D140" s="116" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
@@ -3587,7 +3662,7 @@
       <c r="F151" s="69" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="39" t="inlineStr">
+      <c r="B152" s="121" t="inlineStr">
         <is>
           <t>CRITICAL FAILURE FLAGGED?</t>
         </is>
@@ -3612,7 +3687,7 @@
       <c r="F154" s="68" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="71" t="inlineStr">
+      <c r="B155" s="116" t="inlineStr">
         <is>
           <t>WHAT WENT WELL — behaviors to repeat</t>
         </is>
@@ -3656,7 +3731,7 @@
       <c r="F158" s="69" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="71" t="inlineStr">
+      <c r="B159" s="116" t="inlineStr">
         <is>
           <t>IMPROVEMENT OPPORTUNITIES — behaviors to improve</t>
         </is>
@@ -3700,7 +3775,7 @@
       <c r="F162" s="69" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="71" t="inlineStr">
+      <c r="B163" s="116" t="inlineStr">
         <is>
           <t>COACHING RECOMMENDATION — specific actions the agent should apply going forward</t>
         </is>
@@ -3718,7 +3793,7 @@
       <c r="F164" s="69" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="71" t="inlineStr">
+      <c r="B165" s="116" t="inlineStr">
         <is>
           <t>ORGANIZATIONAL INSIGHTS — training / process / KB / chatbot / tooling / product gaps discovered</t>
         </is>
@@ -3736,7 +3811,7 @@
       <c r="F166" s="69" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="71" t="inlineStr">
+      <c r="B167" s="116" t="inlineStr">
         <is>
           <t>MULTI-TOUCH / JOURNEY NOTES — handoff quality received &amp; passed, continuity, where the chain stands</t>
         </is>
@@ -3754,7 +3829,7 @@
       <c r="F168" s="69" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="71" t="inlineStr">
+      <c r="B169" s="116" t="inlineStr">
         <is>
           <t>FINAL QA ASSESSMENT — customer outcome, support quality, and coaching value</t>
         </is>
@@ -4174,7 +4249,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="104" t="inlineStr">
         <is>
           <t>SCORING GUIDE &amp; CATEGORY CRITERIA</t>
         </is>
@@ -4183,7 +4258,7 @@
       <c r="D1" s="68" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="71" t="inlineStr">
+      <c r="B3" s="116" t="inlineStr">
         <is>
           <t>How to use this form</t>
         </is>
@@ -4264,7 +4339,7 @@
       <c r="D11" s="69" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="71" t="inlineStr">
+      <c r="B13" s="116" t="inlineStr">
         <is>
           <t>Score Anchors (0–5 scale)</t>
         </is>
@@ -4273,12 +4348,12 @@
       <c r="D13" s="68" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="75" t="inlineStr">
+      <c r="B14" s="118" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="C14" s="71" t="inlineStr">
+      <c r="C14" s="116" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -4364,7 +4439,7 @@
       <c r="D20" s="69" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="71" t="inlineStr">
+      <c r="B22" s="116" t="inlineStr">
         <is>
           <t>Indicator ratings</t>
         </is>
@@ -4425,7 +4500,7 @@
       <c r="D26" s="69" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="71" t="inlineStr">
+      <c r="B28" s="116" t="inlineStr">
         <is>
           <t>Category Objectives &amp; Watch-Fors</t>
         </is>
@@ -4525,7 +4600,7 @@
       <c r="D35" s="69" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="71" t="inlineStr">
+      <c r="B37" s="116" t="inlineStr">
         <is>
           <t>Overall Result Bands</t>
         </is>
@@ -4630,7 +4705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C41"/>
+  <dimension ref="B1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4639,7 +4714,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="104" t="inlineStr">
         <is>
           <t>MULTI-TOUCH CASE SCORING — HOW IT WORKS</t>
         </is>
@@ -4647,7 +4722,7 @@
       <c r="C1" s="68" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="71" t="inlineStr">
+      <c r="B3" s="116" t="inlineStr">
         <is>
           <t>THE MECHANICS</t>
         </is>
@@ -4727,7 +4802,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="71" t="inlineStr">
+      <c r="B11" s="116" t="inlineStr">
         <is>
           <t>WORKED JOURNEY — TE00124020 / TE00127492 (Richard &amp; Diana Stell, Linksys WHW03 → MX4200, Apr 1 – May 30, 2026)</t>
         </is>
@@ -4743,12 +4818,12 @@
       <c r="C12" s="69" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="39" t="inlineStr">
+      <c r="B13" s="121" t="inlineStr">
         <is>
           <t>WHERE THE CHAIN BROKE</t>
         </is>
       </c>
-      <c r="C13" s="39" t="inlineStr">
+      <c r="C13" s="121" t="inlineStr">
         <is>
           <t>Scored against the touch that caused it</t>
         </is>
@@ -4839,7 +4914,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="71" t="inlineStr">
+      <c r="B22" s="116" t="inlineStr">
         <is>
           <t>WHERE THE CHAIN RECOVERED (recognize these touches)</t>
         </is>
@@ -4883,7 +4958,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="71" t="inlineStr">
+      <c r="B27" s="116" t="inlineStr">
         <is>
           <t>JOURNEY-LEVEL ORGANIZATIONAL INSIGHTS (do not assign to any single agent's score)</t>
         </is>
@@ -4939,7 +5014,7 @@
       <c r="C33" s="69" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="71" t="inlineStr">
+      <c r="B35" s="116" t="inlineStr">
         <is>
           <t>THE TEAM / JOURNEY SCORE — SCORING THE CHAIN, NOT JUST THE LINKS</t>
         </is>
@@ -5014,9 +5089,60 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="B43" s="125" t="inlineStr">
+        <is>
+          <t>CONTRIBUTION TYPE &amp; HANDOFF QUALITY — PER-TOUCH IMPACT TAGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="46" customHeight="1">
+      <c r="B44" s="52" t="inlineStr">
+        <is>
+          <t>Two extra columns on the Case Tracker (Contribution Type, Handoff Quality) tag what each touch actually did for the case, separately from its category scores. They make the Team Score's Continuity component an informed judgment instead of a guess, and they stop the first agent on a hard case from being penalised for complexity while the last agent gets all the credit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="66" customHeight="1">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Contribution Type (per touch)</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>Resolver = delivered the final fix, correct escalation, or proper closure for that thread · Progress Builder = advanced diagnosis or troubleshooting that moved the case forward, even if not fully fixed · Maintainer = kept momentum, clarified, documented, escalated appropriately without new ground gained · Breaker = reset progress, misdiagnosed, premature closure, or otherwise caused regression. Use 'N/A' only when a touch is purely administrative with no case impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="78" customHeight="1">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Handoff Quality (0-5, per touch)</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Rates the OUTGOING handoff this touch left for whoever (or whatever) came next, across four dimensions: context completeness (did notes explain what was done?), continuity preservation (did it avoid forcing a restart?), expectation alignment (was the customer told something accurate about what happens next?), technical clarity (are logs/findings usable by the next agent?). 5 = clean handoff, nothing to redo · 3-4 = usable with minor gaps · 1-2 = next agent effectively restarts or inherits a broken promise · 0 = handoff itself caused the next failure. Leave blank or mark N/A for a case's final touch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="70" customHeight="1">
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t>Stell journey pattern</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Of the 13 touches, 4 carry Handoff Quality of 1 (Dorothy's wrong callback window, Joziel's 10-15 min promise, Charmaigne's mis-captured email, Riojene's receipt-gate refusal, Jerald's third shifting promise) and 2 are Breaker-tagged for premature RESOLVED closures (Nathan, and via Riojene's refusal). Only Paolo Real and Venn-Emir produced clean Resolver handoffs (4-5). This is what a Continuity score of 1/5 looks like in practice — see the Team Scoring sheet for the live breakdown.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B11:C11"/>
@@ -5029,6 +5155,7 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B43:C43"/>
     <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5041,7 +5168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D58"/>
+  <dimension ref="B1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5056,6 +5183,8 @@
           <t>TEAM SCORING — METHODOLOGY &amp; TEAM OPPORTUNITY ANALYSIS</t>
         </is>
       </c>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="68" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="105" t="inlineStr">
@@ -5063,6 +5192,8 @@
           <t>Individual forms answer 'how did this agent do?'. Team Scoring answers 'how did the CHAIN perform for the customer?' and 'what should we coach, fix, or build as a TEAM?'. The scorecard below is live from the Case Tracker; the worked example is the Stell journey (rows 5-17).</t>
         </is>
       </c>
+      <c r="C2" s="67" t="n"/>
+      <c r="D2" s="68" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="106" t="inlineStr">
@@ -5070,6 +5201,8 @@
           <t>◆  LIVE TEAM SCORECARD  ·  TE00124020 + TE00127492 (Stell Journey)  ◆</t>
         </is>
       </c>
+      <c r="C4" s="126" t="n"/>
+      <c r="D4" s="127" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="107" t="inlineStr">
@@ -5139,6 +5272,8 @@
         <f>" = 50% × "&amp;TEXT('Case Tracker'!D56,"0.0%")&amp;"  +  30% × ("&amp;'Case Tracker'!E56&amp;"÷5)  +  20% × ("&amp;'Case Tracker'!F56&amp;"÷5)  =  "&amp;TEXT('Case Tracker'!G56,"0.0%")&amp;"   (the chain, not just the links)"</f>
         <v/>
       </c>
+      <c r="C9" s="126" t="n"/>
+      <c r="D9" s="127" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="115" t="inlineStr">
@@ -5146,6 +5281,8 @@
           <t>↑ Updates automatically from the Case Tracker (Team/Journey Scores, row 56). Edit Outcome / Continuity there and this scorecard moves with it. For your own journeys, copy this block and point it at the relevant journey row.</t>
         </is>
       </c>
+      <c r="C10" s="70" t="n"/>
+      <c r="D10" s="69" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="116" t="inlineStr">
@@ -5153,6 +5290,8 @@
           <t>1 · WHY A TEAM SCORE EXISTS</t>
         </is>
       </c>
+      <c r="C12" s="67" t="n"/>
+      <c r="D12" s="68" t="n"/>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="B13" s="89" t="inlineStr">
@@ -5160,6 +5299,8 @@
           <t>The rubric's incentive philosophy ranks team improvement FIRST, then individual excellence, then shared accountability. Quality is created collectively — L1, escalation teams, trainers, QA, team leads, operations. A multi-touch case is the truest test: the customer experiences ONE journey, not thirteen separate calls. The Team Score makes the chain itself a scored, coachable unit, so process failures stop hiding between individually 'acceptable' touches. Rule: the Team Score drives team coaching, process fixes, and chain-wide recognition. It is NEVER used for individual discipline — individual feedback comes only from each agent's own touch form.</t>
         </is>
       </c>
+      <c r="C13" s="70" t="n"/>
+      <c r="D13" s="69" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="116" t="inlineStr">
@@ -5167,6 +5308,8 @@
           <t>2 · THE FORMULA, COMPONENT BY COMPONENT</t>
         </is>
       </c>
+      <c r="C15" s="67" t="n"/>
+      <c r="D15" s="68" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="116" t="inlineStr">
@@ -5245,6 +5388,8 @@
           <t>TEAM SCORE  =  50% × 57%  +  30% × (0÷5)  +  20% × (1÷5)  ≈  33%   →   NEEDS IMPROVEMENT   (automatic-review flag also applies: the journey contains critical failures)</t>
         </is>
       </c>
+      <c r="C20" s="67" t="n"/>
+      <c r="D20" s="68" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="116" t="inlineStr">
@@ -5252,6 +5397,8 @@
           <t>3 · READING THE RESULT — THE GAP IS THE DIAGNOSIS</t>
         </is>
       </c>
+      <c r="C22" s="67" t="n"/>
+      <c r="D22" s="68" t="n"/>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="B23" s="88" t="inlineStr">
@@ -5264,6 +5411,7 @@
           <t>The chain neither helped nor hurt. Coach individuals on their own findings; no major process action.</t>
         </is>
       </c>
+      <c r="D23" s="69" t="n"/>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="B24" s="90" t="inlineStr">
@@ -5276,6 +5424,7 @@
           <t>Strong outcome/continuity lifted ordinary touches — the process carried the team. Recognize the chain and the process owners; capture what worked as a standard.</t>
         </is>
       </c>
+      <c r="D24" s="69" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="B25" s="88" t="inlineStr">
@@ -5288,6 +5437,7 @@
           <t>Individually 'acceptable' agents, collectively a lost customer. The failure lives BETWEEN touches: handoffs, statuses, callbacks, ticket linking. Coaching individuals harder will NOT fix this — the action plan must target process, with named owners and dates.</t>
         </is>
       </c>
+      <c r="D25" s="69" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="116" t="inlineStr">
@@ -5295,6 +5445,8 @@
           <t>4 · TEAM CATEGORY HEATMAP — WHERE THE TEAM IS WEAK (live formulas over Case Tracker rows 5-17)</t>
         </is>
       </c>
+      <c r="C27" s="67" t="n"/>
+      <c r="D27" s="68" t="n"/>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="B28" s="98" t="inlineStr">
@@ -5302,6 +5454,8 @@
           <t>Averaging each category ACROSS all touches turns 13 individual reviews into one team profile. Categories below ~2.75 are team-wide coaching themes — they recur regardless of which agent is on the line, so the cause is training, process, or tooling rather than one person.</t>
         </is>
       </c>
+      <c r="C28" s="70" t="n"/>
+      <c r="D28" s="69" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="116" t="inlineStr">
@@ -5438,6 +5592,8 @@
           <t>Reading: red (&lt;2.75) = team coaching theme · yellow (2.75-3.49) = monitor &amp; spot-coach · green (≥3.5) = team strength to protect. Stell profile: a technically capable team losing cases on Ownership, Documentation, and Communication — exactly the 'systemic breakdown in callback management, case ownership, and documentation control' the Concentrix investigation named.</t>
         </is>
       </c>
+      <c r="C37" s="67" t="n"/>
+      <c r="D37" s="68" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="121" t="inlineStr">
@@ -5445,6 +5601,8 @@
           <t>5 · TEAM OPPORTUNITIES IDENTIFIED — STELL JOURNEY (the team action plan)</t>
         </is>
       </c>
+      <c r="C39" s="67" t="n"/>
+      <c r="D39" s="68" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="116" t="inlineStr">
@@ -5605,6 +5763,8 @@
           <t>6 · HOW TO RUN A TEAM REVIEW FOR YOUR OWN JOURNEYS (~30 min once touches are scored)</t>
         </is>
       </c>
+      <c r="C50" s="67" t="n"/>
+      <c r="D50" s="68" t="n"/>
     </row>
     <row r="51" ht="40" customHeight="1">
       <c r="B51" s="122" t="inlineStr">
@@ -5617,6 +5777,7 @@
           <t>Score every touch individually first (Scoring Form per agent) and log all rows in the Case Tracker under the same Case ID.</t>
         </is>
       </c>
+      <c r="D51" s="69" t="n"/>
     </row>
     <row r="52" ht="40" customHeight="1">
       <c r="B52" s="123" t="inlineStr">
@@ -5629,6 +5790,7 @@
           <t>In the Team/Journey Scores section (Case Tracker, row 53+), enter the Case ID — Touches and Avg Touch % auto-fill. Judge Outcome (0-5) and Continuity (0-5) with the anchors in section 2. The Team Score computes; the hero scorecard at the top of this sheet mirrors it.</t>
         </is>
       </c>
+      <c r="D52" s="69" t="n"/>
     </row>
     <row r="53" ht="40" customHeight="1">
       <c r="B53" s="122" t="inlineStr">
@@ -5641,6 +5803,7 @@
           <t>Compare Team Score vs Execution average (section 3). A big negative gap = process problem; flag it as such in your report.</t>
         </is>
       </c>
+      <c r="D53" s="69" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1">
       <c r="B54" s="123" t="inlineStr">
@@ -5653,6 +5816,7 @@
           <t>Build the category heatmap: average each category column across the journey's tracker rows (copy the section-4 formulas, adjusting the row range). Bottom two categories = your team coaching themes.</t>
         </is>
       </c>
+      <c r="D54" s="69" t="n"/>
     </row>
     <row r="55" ht="40" customHeight="1">
       <c r="B55" s="122" t="inlineStr">
@@ -5665,6 +5829,7 @@
           <t>Scan for recurring patterns: same coaching note on 3+ agents (training gap) · same broken-promise type on 2+ touches (process gap) · any premature closure, lost history, or unescalated complaint (critical — name it).</t>
         </is>
       </c>
+      <c r="D55" s="69" t="n"/>
     </row>
     <row r="56" ht="40" customHeight="1">
       <c r="B56" s="123" t="inlineStr">
@@ -5677,6 +5842,7 @@
           <t>Write the team action plan: every opportunity gets an action, a NAMED owner, and a date (section 5 is the model). Recognize the chain's best touches explicitly — including small continuity saves. Deliver individual feedback separately from this team review.</t>
         </is>
       </c>
+      <c r="D56" s="69" t="n"/>
     </row>
     <row r="58" ht="36" customHeight="1">
       <c r="B58" s="93" t="inlineStr">
@@ -5684,10 +5850,240 @@
           <t>Recognition rule: when the Team Score is strong, credit the WHOLE chain — including 2-minute continuity saves like Venn-Emir's email fix. When it is weak despite strong individual touches, the coaching target is the handoff process and its owners, never a hunt for one culprit.</t>
         </is>
       </c>
+      <c r="C58" s="67" t="n"/>
+      <c r="D58" s="68" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="125" t="inlineStr">
+        <is>
+          <t>7 · CONTRIBUTION TYPE &amp; HANDOFF QUALITY — LIVE PER-TOUCH BREAKDOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="B61" s="52" t="inlineStr">
+        <is>
+          <t>Pulled live from the Case Tracker (columns O &amp; P). Use this to judge the Continuity &amp; Handoffs component above — it shows WHERE the chain held and WHERE it broke, touch by touch, instead of one averaged number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="34" customHeight="1">
+      <c r="B62" s="128">
+        <f>"Contribution mix across 13 touches:  "&amp;COUNTIF('Case Tracker'!O5:O17,"Resolver")&amp;" Resolver · "&amp;COUNTIF('Case Tracker'!O5:O17,"Progress Builder")&amp;" Progress Builder · "&amp;COUNTIF('Case Tracker'!O5:O17,"Maintainer")&amp;" Maintainer · "&amp;COUNTIF('Case Tracker'!O5:O17,"Breaker")&amp;" Breaker.   Average Handoff Quality (touches 1-12): "&amp;TEXT(AVERAGE('Case Tracker'!P5:P16),"0.0")&amp;" / 5"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="24" customHeight="1">
+      <c r="B63" s="129" t="inlineStr">
+        <is>
+          <t>Touch (Agent)</t>
+        </is>
+      </c>
+      <c r="C63" s="130" t="inlineStr">
+        <is>
+          <t>Contribution Type</t>
+        </is>
+      </c>
+      <c r="D63" s="130" t="inlineStr">
+        <is>
+          <t>Handoff Quality (0-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="14">
+        <f>'Case Tracker'!D5&amp;" - "&amp;'Case Tracker'!C5</f>
+        <v/>
+      </c>
+      <c r="C64" s="131">
+        <f>'Case Tracker'!O5</f>
+        <v/>
+      </c>
+      <c r="D64" s="131">
+        <f>'Case Tracker'!P5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="12">
+        <f>'Case Tracker'!D6&amp;" - "&amp;'Case Tracker'!C6</f>
+        <v/>
+      </c>
+      <c r="C65" s="132">
+        <f>'Case Tracker'!O6</f>
+        <v/>
+      </c>
+      <c r="D65" s="132">
+        <f>'Case Tracker'!P6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="14">
+        <f>'Case Tracker'!D7&amp;" - "&amp;'Case Tracker'!C7</f>
+        <v/>
+      </c>
+      <c r="C66" s="131">
+        <f>'Case Tracker'!O7</f>
+        <v/>
+      </c>
+      <c r="D66" s="131">
+        <f>'Case Tracker'!P7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="12">
+        <f>'Case Tracker'!D8&amp;" - "&amp;'Case Tracker'!C8</f>
+        <v/>
+      </c>
+      <c r="C67" s="132">
+        <f>'Case Tracker'!O8</f>
+        <v/>
+      </c>
+      <c r="D67" s="132">
+        <f>'Case Tracker'!P8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="14">
+        <f>'Case Tracker'!D9&amp;" - "&amp;'Case Tracker'!C9</f>
+        <v/>
+      </c>
+      <c r="C68" s="131">
+        <f>'Case Tracker'!O9</f>
+        <v/>
+      </c>
+      <c r="D68" s="131">
+        <f>'Case Tracker'!P9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="12">
+        <f>'Case Tracker'!D10&amp;" - "&amp;'Case Tracker'!C10</f>
+        <v/>
+      </c>
+      <c r="C69" s="132">
+        <f>'Case Tracker'!O10</f>
+        <v/>
+      </c>
+      <c r="D69" s="132">
+        <f>'Case Tracker'!P10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="14">
+        <f>'Case Tracker'!D11&amp;" - "&amp;'Case Tracker'!C11</f>
+        <v/>
+      </c>
+      <c r="C70" s="131">
+        <f>'Case Tracker'!O11</f>
+        <v/>
+      </c>
+      <c r="D70" s="131">
+        <f>'Case Tracker'!P11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="12">
+        <f>'Case Tracker'!D12&amp;" - "&amp;'Case Tracker'!C12</f>
+        <v/>
+      </c>
+      <c r="C71" s="132">
+        <f>'Case Tracker'!O12</f>
+        <v/>
+      </c>
+      <c r="D71" s="132">
+        <f>'Case Tracker'!P12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="14">
+        <f>'Case Tracker'!D13&amp;" - "&amp;'Case Tracker'!C13</f>
+        <v/>
+      </c>
+      <c r="C72" s="131">
+        <f>'Case Tracker'!O13</f>
+        <v/>
+      </c>
+      <c r="D72" s="131">
+        <f>'Case Tracker'!P13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="12">
+        <f>'Case Tracker'!D14&amp;" - "&amp;'Case Tracker'!C14</f>
+        <v/>
+      </c>
+      <c r="C73" s="132">
+        <f>'Case Tracker'!O14</f>
+        <v/>
+      </c>
+      <c r="D73" s="132">
+        <f>'Case Tracker'!P14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="14">
+        <f>'Case Tracker'!D15&amp;" - "&amp;'Case Tracker'!C15</f>
+        <v/>
+      </c>
+      <c r="C74" s="131">
+        <f>'Case Tracker'!O15</f>
+        <v/>
+      </c>
+      <c r="D74" s="131">
+        <f>'Case Tracker'!P15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="12">
+        <f>'Case Tracker'!D16&amp;" - "&amp;'Case Tracker'!C16</f>
+        <v/>
+      </c>
+      <c r="C75" s="132">
+        <f>'Case Tracker'!O16</f>
+        <v/>
+      </c>
+      <c r="D75" s="132">
+        <f>'Case Tracker'!P16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="14">
+        <f>'Case Tracker'!D17&amp;" - "&amp;'Case Tracker'!C17</f>
+        <v/>
+      </c>
+      <c r="C76" s="131">
+        <f>'Case Tracker'!O17</f>
+        <v/>
+      </c>
+      <c r="D76" s="131">
+        <f>'Case Tracker'!P17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="B77" s="15" t="inlineStr">
+        <is>
+          <t>Reading this table: a long run of Breaker / low Handoff Quality rows is a process problem (closure discipline, callback management), not an individual one — see Team Opportunities above. A single Breaker surrounded by Resolvers/Progress Builders points at one agent or one moment, and belongs in that agent's individual coaching instead.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="29">
+    <mergeCell ref="B60:D60"/>
     <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B61:D61"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B10:D10"/>
@@ -5695,9 +6091,9 @@
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="C54:D54"/>
     <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="C53:D53"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="C55:D55"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C56:D56"/>
     <mergeCell ref="B20:D20"/>
@@ -5705,7 +6101,9 @@
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="C52:D52"/>
+    <mergeCell ref="B62:D62"/>
     <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B58:D58"/>
@@ -5743,6 +6141,32 @@
     </cfRule>
     <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="0">
       <formula>3.5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C64:C76">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
+      <formula>"Resolver"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="0">
+      <formula>"Progress Builder"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="17">
+      <formula>"Maintainer"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="2">
+      <formula>"Breaker"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D64:D76">
+    <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="between" dxfId="1">
+      <formula>2</formula>
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="15" operator="lessThanOrEqual" dxfId="2">
+      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5790,7 +6214,7 @@
       <c r="F2" s="68" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="71" t="inlineStr">
+      <c r="B4" s="116" t="inlineStr">
         <is>
           <t>1 · CASE INFORMATION</t>
         </is>
@@ -6026,7 +6450,7 @@
       <c r="F16" s="68" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="71" t="inlineStr">
+      <c r="B17" s="116" t="inlineStr">
         <is>
           <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
@@ -6222,7 +6646,7 @@
       <c r="F28" s="69" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="71" t="inlineStr">
+      <c r="B30" s="116" t="inlineStr">
         <is>
           <t>2. TECHNICAL ACCURACY</t>
         </is>
@@ -6456,7 +6880,7 @@
       <c r="F43" s="69" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="B45" s="71" t="inlineStr">
+      <c r="B45" s="116" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
@@ -6709,7 +7133,7 @@
       <c r="F59" s="69" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="B61" s="71" t="inlineStr">
+      <c r="B61" s="116" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
@@ -6962,7 +7386,7 @@
       <c r="F75" s="69" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="B77" s="71" t="inlineStr">
+      <c r="B77" s="116" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
@@ -7158,7 +7582,7 @@
       <c r="F88" s="69" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="B90" s="71" t="inlineStr">
+      <c r="B90" s="116" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
@@ -7373,7 +7797,7 @@
       <c r="F102" s="69" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="B104" s="71" t="inlineStr">
+      <c r="B104" s="116" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
@@ -7618,27 +8042,27 @@
       <c r="F119" s="68" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="75" t="inlineStr">
+      <c r="B120" s="118" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C120" s="75" t="inlineStr">
+      <c r="C120" s="118" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D120" s="75" t="inlineStr">
+      <c r="D120" s="118" t="inlineStr">
         <is>
           <t>Score (0-5)</t>
         </is>
       </c>
-      <c r="E120" s="75" t="inlineStr">
+      <c r="E120" s="118" t="inlineStr">
         <is>
           <t>Weighted</t>
         </is>
       </c>
-      <c r="F120" s="75" t="inlineStr">
+      <c r="F120" s="118" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
@@ -7819,7 +8243,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="71" t="inlineStr">
+      <c r="B130" s="116" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
@@ -7875,7 +8299,7 @@
       <c r="F133" s="69" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="71" t="inlineStr">
+      <c r="B135" s="116" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
@@ -7923,7 +8347,7 @@
       <c r="F137" s="69" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="39" t="inlineStr">
+      <c r="B139" s="121" t="inlineStr">
         <is>
           <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
         </is>
@@ -7934,17 +8358,17 @@
       <c r="F139" s="68" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="71" t="inlineStr">
+      <c r="B140" s="116" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="C140" s="75" t="inlineStr">
+      <c r="C140" s="118" t="inlineStr">
         <is>
           <t>Present?</t>
         </is>
       </c>
-      <c r="D140" s="71" t="inlineStr">
+      <c r="D140" s="116" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
@@ -8130,7 +8554,7 @@
       <c r="F151" s="69" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="39" t="inlineStr">
+      <c r="B152" s="121" t="inlineStr">
         <is>
           <t>CRITICAL FAILURE FLAGGED?</t>
         </is>
@@ -8155,7 +8579,7 @@
       <c r="F154" s="68" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="71" t="inlineStr">
+      <c r="B155" s="116" t="inlineStr">
         <is>
           <t>WHAT WENT WELL — behaviors to repeat</t>
         </is>
@@ -8211,7 +8635,7 @@
       <c r="F158" s="69" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="71" t="inlineStr">
+      <c r="B159" s="116" t="inlineStr">
         <is>
           <t>IMPROVEMENT OPPORTUNITIES — behaviors to improve</t>
         </is>
@@ -8267,7 +8691,7 @@
       <c r="F162" s="69" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="71" t="inlineStr">
+      <c r="B163" s="116" t="inlineStr">
         <is>
           <t>COACHING RECOMMENDATION — specific actions the agent should apply going forward</t>
         </is>
@@ -8289,7 +8713,7 @@
       <c r="F164" s="69" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="71" t="inlineStr">
+      <c r="B165" s="116" t="inlineStr">
         <is>
           <t>ORGANIZATIONAL INSIGHTS — training / process / KB / chatbot / tooling / product gaps discovered</t>
         </is>
@@ -8311,7 +8735,7 @@
       <c r="F166" s="69" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="71" t="inlineStr">
+      <c r="B167" s="116" t="inlineStr">
         <is>
           <t>MULTI-TOUCH / JOURNEY NOTES — handoff quality received &amp; passed, continuity, where the chain stands</t>
         </is>
@@ -8333,7 +8757,7 @@
       <c r="F168" s="69" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="71" t="inlineStr">
+      <c r="B169" s="116" t="inlineStr">
         <is>
           <t>FINAL QA ASSESSMENT — customer outcome, support quality, and coaching value</t>
         </is>
@@ -8747,7 +9171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8764,10 +9188,12 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="104" t="inlineStr">
         <is>
           <t>CASE TRACKER — Multi-Case &amp; Multi-Touch Log</t>
         </is>
@@ -8784,7 +9210,9 @@
       <c r="K1" s="67" t="n"/>
       <c r="L1" s="67" t="n"/>
       <c r="M1" s="67" t="n"/>
-      <c r="N1" s="68" t="n"/>
+      <c r="N1" s="67" t="n"/>
+      <c r="O1" s="67" t="n"/>
+      <c r="P1" s="68" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="59" t="inlineStr">
@@ -8804,15 +9232,32 @@
       <c r="K2" s="67" t="n"/>
       <c r="L2" s="67" t="n"/>
       <c r="M2" s="67" t="n"/>
-      <c r="N2" s="68" t="n"/>
+      <c r="N2" s="67" t="n"/>
+      <c r="O2" s="67" t="n"/>
+      <c r="P2" s="68" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="124">
         <f>" LOADED JOURNEY TEAM SCORE  ▸  TE00127492 (Stell):  "&amp;TEXT(G56,"0.0%")&amp;"   "&amp;UPPER(H56)&amp;"     —  full team analysis on the Team Scoring sheet;  scoring section below at row 53 "</f>
         <v/>
       </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
+      <c r="B3" s="67" t="n"/>
+      <c r="C3" s="67" t="n"/>
+      <c r="D3" s="67" t="n"/>
+      <c r="E3" s="67" t="n"/>
+      <c r="F3" s="67" t="n"/>
+      <c r="G3" s="67" t="n"/>
+      <c r="H3" s="67" t="n"/>
+      <c r="I3" s="67" t="n"/>
+      <c r="J3" s="67" t="n"/>
+      <c r="K3" s="67" t="n"/>
+      <c r="L3" s="67" t="n"/>
+      <c r="M3" s="67" t="n"/>
+      <c r="N3" s="67" t="n"/>
+      <c r="O3" s="67" t="n"/>
+      <c r="P3" s="68" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="60" t="inlineStr">
         <is>
           <t>Date</t>
@@ -8881,6 +9326,16 @@
       <c r="N4" s="60" t="inlineStr">
         <is>
           <t>Outcome / Notes</t>
+        </is>
+      </c>
+      <c r="O4" s="130" t="inlineStr">
+        <is>
+          <t>Contribution Type</t>
+        </is>
+      </c>
+      <c r="P4" s="130" t="inlineStr">
+        <is>
+          <t>Handoff Quality (0-5)</t>
         </is>
       </c>
     </row>
@@ -8937,6 +9392,14 @@
           <t>$30 paid session (76m): node power isolation, error 2298, escalated to L2. CRITICAL: card data spoken aloud (PCI) + $30 charge never documented. Promised 2-3h callback vs 24-48h process.</t>
         </is>
       </c>
+      <c r="O5" s="132" t="inlineStr">
+        <is>
+          <t>Progress Builder</t>
+        </is>
+      </c>
+      <c r="P5" s="132" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="61" t="inlineStr">
@@ -8991,6 +9454,14 @@
           <t>Follow-up: no callback received, household offline. Promised L2 callback in 10-15 min without naming a technician. Administrative only.</t>
         </is>
       </c>
+      <c r="O6" s="131" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="P6" s="131" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="61" t="inlineStr">
@@ -9045,6 +9516,14 @@
           <t>Delayed L2 callback (4h, internal 'weekly meeting' excuse) but RESTORED Wi-Fi: recovery key, admin reset, new SSID. Comm gaps: pace, terminology, hearing adaptation.</t>
         </is>
       </c>
+      <c r="O7" s="132" t="inlineStr">
+        <is>
+          <t>Resolver</t>
+        </is>
+      </c>
+      <c r="P7" s="132" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="61" t="inlineStr">
@@ -9099,6 +9578,14 @@
           <t>88-min session on drop cycles: 2 child nodes restored via reset/re-add; 1 node unstable at end. Solid effort; instructions too compound for the customer.</t>
         </is>
       </c>
+      <c r="O8" s="131" t="inlineStr">
+        <is>
+          <t>Progress Builder</t>
+        </is>
+      </c>
+      <c r="P8" s="131" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
@@ -9153,6 +9640,14 @@
           <t>WHW03 no-light call: warranty check, child-node-as-parent advice, self-help email offered. Email address mis-captured despite phonetic spelling → promised guide never arrived.</t>
         </is>
       </c>
+      <c r="O9" s="132" t="inlineStr">
+        <is>
+          <t>Maintainer</t>
+        </is>
+      </c>
+      <c r="P9" s="132" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="61" t="inlineStr">
@@ -9207,6 +9702,14 @@
           <t>Caught and corrected the wrong email in under 2 min, re-sent guide. Clean recovery; investigation: no opportunities observed.</t>
         </is>
       </c>
+      <c r="O10" s="131" t="inlineStr">
+        <is>
+          <t>Resolver</t>
+        </is>
+      </c>
+      <c r="P10" s="131" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="61" t="inlineStr">
@@ -9261,6 +9764,14 @@
           <t>100-min MX4200 setup (3 new + old nodes). Marked RESOLVED 10 min after note; issue returned in 3 days. CRITICAL: premature closure. Hearing adaptation cited 8×.</t>
         </is>
       </c>
+      <c r="O11" s="132" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="P11" s="132" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="61" t="inlineStr">
@@ -9315,6 +9826,14 @@
           <t>Active 5-min drop cycles, but troubleshooting refused pending warranty receipt; note: 'No trouble shooting made.' Receipt-gate replaced support on an active issue.</t>
         </is>
       </c>
+      <c r="O12" s="131" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="P12" s="131" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
@@ -9369,6 +9888,14 @@
           <t>Channel Finder, firmware, RSSI (-62/-71), sequence reboot, logs collected. Ended 'observe 1 hour' + RESOLVED again; note says 'cx appreciate the help' masking exhaustion.</t>
         </is>
       </c>
+      <c r="O13" s="132" t="inlineStr">
+        <is>
+          <t>Progress Builder</t>
+        </is>
+      </c>
+      <c r="P13" s="132" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="61" t="inlineStr">
@@ -9423,6 +9950,14 @@
           <t>Repeated power-cycle the customer had already done; -76 dBm clue not isolated. Escalation to L2 appropriate; callback expectation changed 24h → 2h. Understated contact count (4 vs 7+).</t>
         </is>
       </c>
+      <c r="O14" s="131" t="inlineStr">
+        <is>
+          <t>Maintainer</t>
+        </is>
+      </c>
+      <c r="P14" s="131" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="61" t="inlineStr">
@@ -9477,6 +10012,14 @@
           <t>Best diagnostics of journey (98m): HomeKit isolation, AT&amp;T SSID interference theory, firmware validation, sysinfo logs captured, 2 bad nodes (-90/-93 dBm), L2 hotline given. Still closed RESOLVED on an observed-only state.</t>
         </is>
       </c>
+      <c r="O15" s="132" t="inlineStr">
+        <is>
+          <t>Progress Builder</t>
+        </is>
+      </c>
+      <c r="P15" s="132" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="61" t="inlineStr">
@@ -9531,6 +10074,14 @@
           <t>Customer 3+ hours into wait, third shifting callback promise of the day. Did re-escalate with CAT approval. No fallback plan offered; customer: 'I don't believe anything I've been told today.'</t>
         </is>
       </c>
+      <c r="O16" s="131" t="inlineStr">
+        <is>
+          <t>Maintainer</t>
+        </is>
+      </c>
+      <c r="P16" s="131" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="61" t="inlineStr">
@@ -9583,6 +10134,16 @@
       <c r="N17" s="12" t="inlineStr">
         <is>
           <t>FINAL TOUCH — full form on Example (Filled). 3h26m session restored internet (482-530 Mbps), 4 child nodes + RSSI documented. Then: agreed 4-5 PM callback missed by 42-66 min; RESOLVED with no closure note; management/legal request not escalated. CSAT 1/5; customer switched to Eero.</t>
+        </is>
+      </c>
+      <c r="O17" s="132" t="inlineStr">
+        <is>
+          <t>Resolver</t>
+        </is>
+      </c>
+      <c r="P17" s="132" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -9607,6 +10168,8 @@
         <v/>
       </c>
       <c r="N18" s="14" t="inlineStr"/>
+      <c r="O18" s="131" t="inlineStr"/>
+      <c r="P18" s="131" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="61" t="inlineStr"/>
@@ -9629,6 +10192,8 @@
         <v/>
       </c>
       <c r="N19" s="12" t="inlineStr"/>
+      <c r="O19" s="132" t="inlineStr"/>
+      <c r="P19" s="132" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="61" t="inlineStr"/>
@@ -9651,6 +10216,8 @@
         <v/>
       </c>
       <c r="N20" s="14" t="inlineStr"/>
+      <c r="O20" s="131" t="inlineStr"/>
+      <c r="P20" s="131" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="61" t="inlineStr"/>
@@ -9673,6 +10240,8 @@
         <v/>
       </c>
       <c r="N21" s="12" t="inlineStr"/>
+      <c r="O21" s="132" t="inlineStr"/>
+      <c r="P21" s="132" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="61" t="inlineStr"/>
@@ -9695,6 +10264,8 @@
         <v/>
       </c>
       <c r="N22" s="14" t="inlineStr"/>
+      <c r="O22" s="131" t="inlineStr"/>
+      <c r="P22" s="131" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="61" t="inlineStr"/>
@@ -9717,6 +10288,8 @@
         <v/>
       </c>
       <c r="N23" s="12" t="inlineStr"/>
+      <c r="O23" s="132" t="inlineStr"/>
+      <c r="P23" s="132" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="61" t="inlineStr"/>
@@ -9739,6 +10312,8 @@
         <v/>
       </c>
       <c r="N24" s="14" t="inlineStr"/>
+      <c r="O24" s="131" t="inlineStr"/>
+      <c r="P24" s="131" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="61" t="inlineStr"/>
@@ -9761,6 +10336,8 @@
         <v/>
       </c>
       <c r="N25" s="12" t="inlineStr"/>
+      <c r="O25" s="132" t="inlineStr"/>
+      <c r="P25" s="132" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="61" t="inlineStr"/>
@@ -9783,6 +10360,8 @@
         <v/>
       </c>
       <c r="N26" s="14" t="inlineStr"/>
+      <c r="O26" s="131" t="inlineStr"/>
+      <c r="P26" s="131" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="61" t="inlineStr"/>
@@ -9805,6 +10384,8 @@
         <v/>
       </c>
       <c r="N27" s="12" t="inlineStr"/>
+      <c r="O27" s="132" t="inlineStr"/>
+      <c r="P27" s="132" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="61" t="inlineStr"/>
@@ -9827,6 +10408,8 @@
         <v/>
       </c>
       <c r="N28" s="14" t="inlineStr"/>
+      <c r="O28" s="131" t="inlineStr"/>
+      <c r="P28" s="131" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="61" t="inlineStr"/>
@@ -9849,6 +10432,8 @@
         <v/>
       </c>
       <c r="N29" s="12" t="inlineStr"/>
+      <c r="O29" s="132" t="inlineStr"/>
+      <c r="P29" s="132" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="61" t="inlineStr"/>
@@ -9871,6 +10456,8 @@
         <v/>
       </c>
       <c r="N30" s="14" t="inlineStr"/>
+      <c r="O30" s="131" t="inlineStr"/>
+      <c r="P30" s="131" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="61" t="inlineStr"/>
@@ -9893,6 +10480,8 @@
         <v/>
       </c>
       <c r="N31" s="12" t="inlineStr"/>
+      <c r="O31" s="132" t="inlineStr"/>
+      <c r="P31" s="132" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="61" t="inlineStr"/>
@@ -9915,6 +10504,8 @@
         <v/>
       </c>
       <c r="N32" s="14" t="inlineStr"/>
+      <c r="O32" s="131" t="inlineStr"/>
+      <c r="P32" s="131" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="61" t="inlineStr"/>
@@ -9937,6 +10528,8 @@
         <v/>
       </c>
       <c r="N33" s="12" t="inlineStr"/>
+      <c r="O33" s="132" t="inlineStr"/>
+      <c r="P33" s="132" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="61" t="inlineStr"/>
@@ -9959,6 +10552,8 @@
         <v/>
       </c>
       <c r="N34" s="14" t="inlineStr"/>
+      <c r="O34" s="131" t="inlineStr"/>
+      <c r="P34" s="131" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="61" t="inlineStr"/>
@@ -9981,6 +10576,8 @@
         <v/>
       </c>
       <c r="N35" s="12" t="inlineStr"/>
+      <c r="O35" s="132" t="inlineStr"/>
+      <c r="P35" s="132" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="61" t="inlineStr"/>
@@ -10003,6 +10600,8 @@
         <v/>
       </c>
       <c r="N36" s="14" t="inlineStr"/>
+      <c r="O36" s="131" t="inlineStr"/>
+      <c r="P36" s="131" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="61" t="inlineStr"/>
@@ -10025,6 +10624,8 @@
         <v/>
       </c>
       <c r="N37" s="12" t="inlineStr"/>
+      <c r="O37" s="132" t="inlineStr"/>
+      <c r="P37" s="132" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="61" t="inlineStr"/>
@@ -10047,6 +10648,8 @@
         <v/>
       </c>
       <c r="N38" s="14" t="inlineStr"/>
+      <c r="O38" s="131" t="inlineStr"/>
+      <c r="P38" s="131" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="61" t="inlineStr"/>
@@ -10069,6 +10672,8 @@
         <v/>
       </c>
       <c r="N39" s="12" t="inlineStr"/>
+      <c r="O39" s="132" t="inlineStr"/>
+      <c r="P39" s="132" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="61" t="inlineStr"/>
@@ -10091,6 +10696,8 @@
         <v/>
       </c>
       <c r="N40" s="14" t="inlineStr"/>
+      <c r="O40" s="131" t="inlineStr"/>
+      <c r="P40" s="131" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="61" t="inlineStr"/>
@@ -10113,6 +10720,8 @@
         <v/>
       </c>
       <c r="N41" s="12" t="inlineStr"/>
+      <c r="O41" s="132" t="inlineStr"/>
+      <c r="P41" s="132" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="61" t="inlineStr"/>
@@ -10135,6 +10744,8 @@
         <v/>
       </c>
       <c r="N42" s="14" t="inlineStr"/>
+      <c r="O42" s="131" t="inlineStr"/>
+      <c r="P42" s="131" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="61" t="inlineStr"/>
@@ -10157,6 +10768,8 @@
         <v/>
       </c>
       <c r="N43" s="12" t="inlineStr"/>
+      <c r="O43" s="132" t="inlineStr"/>
+      <c r="P43" s="132" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="61" t="inlineStr"/>
@@ -10179,6 +10792,8 @@
         <v/>
       </c>
       <c r="N44" s="14" t="inlineStr"/>
+      <c r="O44" s="131" t="inlineStr"/>
+      <c r="P44" s="131" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="61" t="inlineStr"/>
@@ -10201,6 +10816,8 @@
         <v/>
       </c>
       <c r="N45" s="12" t="inlineStr"/>
+      <c r="O45" s="132" t="inlineStr"/>
+      <c r="P45" s="132" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="61" t="inlineStr"/>
@@ -10223,6 +10840,8 @@
         <v/>
       </c>
       <c r="N46" s="14" t="inlineStr"/>
+      <c r="O46" s="131" t="inlineStr"/>
+      <c r="P46" s="131" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="61" t="inlineStr"/>
@@ -10245,6 +10864,8 @@
         <v/>
       </c>
       <c r="N47" s="12" t="inlineStr"/>
+      <c r="O47" s="132" t="inlineStr"/>
+      <c r="P47" s="132" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="61" t="inlineStr"/>
@@ -10267,6 +10888,8 @@
         <v/>
       </c>
       <c r="N48" s="14" t="inlineStr"/>
+      <c r="O48" s="131" t="inlineStr"/>
+      <c r="P48" s="131" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="61" t="inlineStr"/>
@@ -10289,6 +10912,8 @@
         <v/>
       </c>
       <c r="N49" s="12" t="inlineStr"/>
+      <c r="O49" s="132" t="inlineStr"/>
+      <c r="P49" s="132" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -10356,7 +10981,9 @@
       <c r="K53" s="67" t="n"/>
       <c r="L53" s="67" t="n"/>
       <c r="M53" s="67" t="n"/>
-      <c r="N53" s="68" t="n"/>
+      <c r="N53" s="67" t="n"/>
+      <c r="O53" s="67" t="n"/>
+      <c r="P53" s="68" t="n"/>
     </row>
     <row r="54" ht="32" customHeight="1">
       <c r="A54" s="74" t="inlineStr">
@@ -10376,16 +11003,18 @@
       <c r="K54" s="67" t="n"/>
       <c r="L54" s="67" t="n"/>
       <c r="M54" s="67" t="n"/>
-      <c r="N54" s="68" t="n"/>
+      <c r="N54" s="67" t="n"/>
+      <c r="O54" s="67" t="n"/>
+      <c r="P54" s="68" t="n"/>
     </row>
     <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="75" t="inlineStr">
+      <c r="A55" s="118" t="inlineStr">
         <is>
           <t>Journey / Case ID(s)</t>
         </is>
       </c>
       <c r="B55" s="68" t="n"/>
-      <c r="C55" s="75" t="inlineStr">
+      <c r="C55" s="118" t="inlineStr">
         <is>
           <t>Touches</t>
         </is>
@@ -10410,12 +11039,12 @@
           <t>TEAM SCORE</t>
         </is>
       </c>
-      <c r="H55" s="75" t="inlineStr">
+      <c r="H55" s="118" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="I55" s="71" t="inlineStr">
+      <c r="I55" s="116" t="inlineStr">
         <is>
           <t>Journey notes (where the chain broke / recovered)</t>
         </is>
@@ -10572,23 +11201,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="I57:N57"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A53:N53"/>
-    <mergeCell ref="I55:N55"/>
     <mergeCell ref="A59:B59"/>
     <mergeCell ref="A57:B57"/>
     <mergeCell ref="I59:N59"/>
-    <mergeCell ref="A54:N54"/>
-    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A53:P53"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A60:N60"/>
+    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="I58:N58"/>
+    <mergeCell ref="I55:N55"/>
+    <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="I58:N58"/>
+    <mergeCell ref="I57:N57"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <conditionalFormatting sqref="L5:L49">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
@@ -10650,7 +11279,33 @@
       <formula>$G$56&lt;0.7</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <conditionalFormatting sqref="O5:O49">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="0">
+      <formula>"Resolver"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="0">
+      <formula>"Progress Builder"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="17">
+      <formula>"Maintainer"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="2">
+      <formula>"Breaker"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P49">
+    <cfRule type="cellIs" priority="21" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="between" dxfId="1">
+      <formula>2</formula>
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="23" operator="lessThanOrEqual" dxfId="2">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation sqref="E5:K5 E6:K6 E7:K7 E8:K8 E9:K9 E10:K10 E11:K11 E12:K12 E13:K13 E14:K14 E15:K15 E16:K16 E17:K17 E18:K18 E19:K19 E20:K20 E21:K21 E22:K22 E23:K23 E24:K24 E25:K25 E26:K26 E27:K27 E28:K28 E29:K29 E30:K30 E31:K31 E32:K32 E33:K33 E34:K34 E35:K35 E36:K36 E37:K37 E38:K38 E39:K39 E40:K40 E41:K41 E42:K42 E43:K43 E44:K44 E45:K45 E46:K46 E47:K47 E48:K48 E49:K49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>5</formula2>
@@ -10659,6 +11314,13 @@
       <formula1>0</formula1>
       <formula2>5</formula2>
     </dataValidation>
+    <dataValidation sqref="O5:O49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Resolver, Progress Builder, Maintainer, Breaker, or N/A." type="list">
+      <formula1>"Resolver,Progress Builder,Maintainer,Breaker,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename Contribution Type "Breaker" to "Regression Contributor"
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form.xlsx
+++ b/QA Scoring Form.xlsx
@@ -1828,7 +1828,7 @@
       <c r="F2" s="68" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="116" t="inlineStr">
+      <c r="B4" s="125" t="inlineStr">
         <is>
           <t>1 · CASE INFORMATION</t>
         </is>
@@ -1992,7 +1992,7 @@
       <c r="F16" s="68" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="116" t="inlineStr">
+      <c r="B17" s="125" t="inlineStr">
         <is>
           <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
@@ -2142,7 +2142,7 @@
       <c r="F28" s="69" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="116" t="inlineStr">
+      <c r="B30" s="125" t="inlineStr">
         <is>
           <t>2. TECHNICAL ACCURACY</t>
         </is>
@@ -2314,7 +2314,7 @@
       <c r="F43" s="69" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="B45" s="116" t="inlineStr">
+      <c r="B45" s="125" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
@@ -2497,7 +2497,7 @@
       <c r="F59" s="69" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="B61" s="116" t="inlineStr">
+      <c r="B61" s="125" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
@@ -2680,7 +2680,7 @@
       <c r="F75" s="69" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="B77" s="116" t="inlineStr">
+      <c r="B77" s="125" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
@@ -2830,7 +2830,7 @@
       <c r="F88" s="69" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="B90" s="116" t="inlineStr">
+      <c r="B90" s="125" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
@@ -2991,7 +2991,7 @@
       <c r="F102" s="69" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="B104" s="116" t="inlineStr">
+      <c r="B104" s="125" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
@@ -3217,7 +3217,7 @@
         <f>IF(D121="","",(D121/5)*C121)</f>
         <v/>
       </c>
-      <c r="F121" s="82">
+      <c r="F121" s="132">
         <f>IF(D121="","",IF(D121&gt;=4,"Strong",IF(D121=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3239,7 +3239,7 @@
         <f>IF(D122="","",(D122/5)*C122)</f>
         <v/>
       </c>
-      <c r="F122" s="77">
+      <c r="F122" s="131">
         <f>IF(D122="","",IF(D122&gt;=4,"Strong",IF(D122=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3261,7 +3261,7 @@
         <f>IF(D123="","",(D123/5)*C123)</f>
         <v/>
       </c>
-      <c r="F123" s="82">
+      <c r="F123" s="132">
         <f>IF(D123="","",IF(D123&gt;=4,"Strong",IF(D123=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3283,7 +3283,7 @@
         <f>IF(D124="","",(D124/5)*C124)</f>
         <v/>
       </c>
-      <c r="F124" s="77">
+      <c r="F124" s="131">
         <f>IF(D124="","",IF(D124&gt;=4,"Strong",IF(D124=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3305,7 +3305,7 @@
         <f>IF(D125="","",(D125/5)*C125)</f>
         <v/>
       </c>
-      <c r="F125" s="82">
+      <c r="F125" s="132">
         <f>IF(D125="","",IF(D125&gt;=4,"Strong",IF(D125=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3327,7 +3327,7 @@
         <f>IF(D126="","",(D126/5)*C126)</f>
         <v/>
       </c>
-      <c r="F126" s="77">
+      <c r="F126" s="131">
         <f>IF(D126="","",IF(D126&gt;=4,"Strong",IF(D126=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3349,7 +3349,7 @@
         <f>IF(D127="","",(D127/5)*C127)</f>
         <v/>
       </c>
-      <c r="F127" s="82">
+      <c r="F127" s="132">
         <f>IF(D127="","",IF(D127&gt;=4,"Strong",IF(D127=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -3375,7 +3375,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="116" t="inlineStr">
+      <c r="B130" s="125" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
@@ -3419,7 +3419,7 @@
       <c r="F133" s="69" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="116" t="inlineStr">
+      <c r="B135" s="125" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
@@ -3478,7 +3478,7 @@
       <c r="F139" s="68" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="116" t="inlineStr">
+      <c r="B140" s="125" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
@@ -3488,7 +3488,7 @@
           <t>Present?</t>
         </is>
       </c>
-      <c r="D140" s="116" t="inlineStr">
+      <c r="D140" s="125" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
@@ -3687,7 +3687,7 @@
       <c r="F154" s="68" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="116" t="inlineStr">
+      <c r="B155" s="125" t="inlineStr">
         <is>
           <t>WHAT WENT WELL — behaviors to repeat</t>
         </is>
@@ -3731,7 +3731,7 @@
       <c r="F158" s="69" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="116" t="inlineStr">
+      <c r="B159" s="125" t="inlineStr">
         <is>
           <t>IMPROVEMENT OPPORTUNITIES — behaviors to improve</t>
         </is>
@@ -3775,7 +3775,7 @@
       <c r="F162" s="69" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="116" t="inlineStr">
+      <c r="B163" s="125" t="inlineStr">
         <is>
           <t>COACHING RECOMMENDATION — specific actions the agent should apply going forward</t>
         </is>
@@ -3793,7 +3793,7 @@
       <c r="F164" s="69" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="116" t="inlineStr">
+      <c r="B165" s="125" t="inlineStr">
         <is>
           <t>ORGANIZATIONAL INSIGHTS — training / process / KB / chatbot / tooling / product gaps discovered</t>
         </is>
@@ -3811,7 +3811,7 @@
       <c r="F166" s="69" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="116" t="inlineStr">
+      <c r="B167" s="125" t="inlineStr">
         <is>
           <t>MULTI-TOUCH / JOURNEY NOTES — handoff quality received &amp; passed, continuity, where the chain stands</t>
         </is>
@@ -3829,7 +3829,7 @@
       <c r="F168" s="69" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="116" t="inlineStr">
+      <c r="B169" s="125" t="inlineStr">
         <is>
           <t>FINAL QA ASSESSMENT — customer outcome, support quality, and coaching value</t>
         </is>
@@ -4258,7 +4258,7 @@
       <c r="D1" s="68" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="116" t="inlineStr">
+      <c r="B3" s="125" t="inlineStr">
         <is>
           <t>How to use this form</t>
         </is>
@@ -4339,7 +4339,7 @@
       <c r="D11" s="69" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="116" t="inlineStr">
+      <c r="B13" s="125" t="inlineStr">
         <is>
           <t>Score Anchors (0–5 scale)</t>
         </is>
@@ -4353,7 +4353,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="C14" s="116" t="inlineStr">
+      <c r="C14" s="125" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -4439,7 +4439,7 @@
       <c r="D20" s="69" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="116" t="inlineStr">
+      <c r="B22" s="125" t="inlineStr">
         <is>
           <t>Indicator ratings</t>
         </is>
@@ -4500,7 +4500,7 @@
       <c r="D26" s="69" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="116" t="inlineStr">
+      <c r="B28" s="125" t="inlineStr">
         <is>
           <t>Category Objectives &amp; Watch-Fors</t>
         </is>
@@ -4600,7 +4600,7 @@
       <c r="D35" s="69" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="116" t="inlineStr">
+      <c r="B37" s="125" t="inlineStr">
         <is>
           <t>Overall Result Bands</t>
         </is>
@@ -4722,7 +4722,7 @@
       <c r="C1" s="68" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="116" t="inlineStr">
+      <c r="B3" s="125" t="inlineStr">
         <is>
           <t>THE MECHANICS</t>
         </is>
@@ -4802,7 +4802,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="116" t="inlineStr">
+      <c r="B11" s="125" t="inlineStr">
         <is>
           <t>WORKED JOURNEY — TE00124020 / TE00127492 (Richard &amp; Diana Stell, Linksys WHW03 → MX4200, Apr 1 – May 30, 2026)</t>
         </is>
@@ -4914,7 +4914,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="116" t="inlineStr">
+      <c r="B22" s="125" t="inlineStr">
         <is>
           <t>WHERE THE CHAIN RECOVERED (recognize these touches)</t>
         </is>
@@ -4958,7 +4958,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="116" t="inlineStr">
+      <c r="B27" s="125" t="inlineStr">
         <is>
           <t>JOURNEY-LEVEL ORGANIZATIONAL INSIGHTS (do not assign to any single agent's score)</t>
         </is>
@@ -5014,7 +5014,7 @@
       <c r="C33" s="69" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="116" t="inlineStr">
+      <c r="B35" s="125" t="inlineStr">
         <is>
           <t>THE TEAM / JOURNEY SCORE — SCORING THE CHAIN, NOT JUST THE LINKS</t>
         </is>
@@ -5095,6 +5095,7 @@
           <t>CONTRIBUTION TYPE &amp; HANDOFF QUALITY — PER-TOUCH IMPACT TAGS</t>
         </is>
       </c>
+      <c r="C43" s="68" t="n"/>
     </row>
     <row r="44" ht="46" customHeight="1">
       <c r="B44" s="52" t="inlineStr">
@@ -5102,6 +5103,7 @@
           <t>Two extra columns on the Case Tracker (Contribution Type, Handoff Quality) tag what each touch actually did for the case, separately from its category scores. They make the Team Score's Continuity component an informed judgment instead of a guess, and they stop the first agent on a hard case from being penalised for complexity while the last agent gets all the credit.</t>
         </is>
       </c>
+      <c r="C44" s="68" t="n"/>
     </row>
     <row r="45" ht="66" customHeight="1">
       <c r="B45" s="44" t="inlineStr">
@@ -5111,7 +5113,7 @@
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Resolver = delivered the final fix, correct escalation, or proper closure for that thread · Progress Builder = advanced diagnosis or troubleshooting that moved the case forward, even if not fully fixed · Maintainer = kept momentum, clarified, documented, escalated appropriately without new ground gained · Breaker = reset progress, misdiagnosed, premature closure, or otherwise caused regression. Use 'N/A' only when a touch is purely administrative with no case impact.</t>
+          <t>Resolver = delivered the final fix, correct escalation, or proper closure for that thread · Progress Builder = advanced diagnosis or troubleshooting that moved the case forward, even if not fully fixed · Maintainer = kept momentum, clarified, documented, escalated appropriately without new ground gained · Regression Contributor = reset progress, misdiagnosed, premature closure, or otherwise caused regression. Use 'N/A' only when a touch is purely administrative with no case impact.</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5137,7 @@
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Of the 13 touches, 4 carry Handoff Quality of 1 (Dorothy's wrong callback window, Joziel's 10-15 min promise, Charmaigne's mis-captured email, Riojene's receipt-gate refusal, Jerald's third shifting promise) and 2 are Breaker-tagged for premature RESOLVED closures (Nathan, and via Riojene's refusal). Only Paolo Real and Venn-Emir produced clean Resolver handoffs (4-5). This is what a Continuity score of 1/5 looks like in practice — see the Team Scoring sheet for the live breakdown.</t>
+          <t>Of the 13 touches, 4 carry Handoff Quality of 1 (Dorothy's wrong callback window, Joziel's 10-15 min promise, Charmaigne's mis-captured email, Riojene's receipt-gate refusal, Jerald's third shifting promise) and 2 are Regression Contributor-tagged for premature RESOLVED closures (Nathan, and via Riojene's refusal). Only Paolo Real and Venn-Emir produced clean Resolver handoffs (4-5). This is what a Continuity score of 1/5 looks like in practice — see the Team Scoring sheet for the live breakdown.</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5287,7 @@
       <c r="D10" s="69" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="116" t="inlineStr">
+      <c r="B12" s="125" t="inlineStr">
         <is>
           <t>1 · WHY A TEAM SCORE EXISTS</t>
         </is>
@@ -5303,7 +5305,7 @@
       <c r="D13" s="69" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="116" t="inlineStr">
+      <c r="B15" s="125" t="inlineStr">
         <is>
           <t>2 · THE FORMULA, COMPONENT BY COMPONENT</t>
         </is>
@@ -5312,17 +5314,17 @@
       <c r="D15" s="68" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="116" t="inlineStr">
+      <c r="B16" s="125" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C16" s="116" t="inlineStr">
+      <c r="C16" s="125" t="inlineStr">
         <is>
           <t>What it measures &amp; why this weight</t>
         </is>
       </c>
-      <c r="D16" s="116" t="inlineStr">
+      <c r="D16" s="125" t="inlineStr">
         <is>
           <t>Stell journey worked numbers</t>
         </is>
@@ -5392,7 +5394,7 @@
       <c r="D20" s="68" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="116" t="inlineStr">
+      <c r="B22" s="125" t="inlineStr">
         <is>
           <t>3 · READING THE RESULT — THE GAP IS THE DIAGNOSIS</t>
         </is>
@@ -5440,7 +5442,7 @@
       <c r="D25" s="69" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="116" t="inlineStr">
+      <c r="B27" s="125" t="inlineStr">
         <is>
           <t>4 · TEAM CATEGORY HEATMAP — WHERE THE TEAM IS WEAK (live formulas over Case Tracker rows 5-17)</t>
         </is>
@@ -5458,7 +5460,7 @@
       <c r="D28" s="69" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="116" t="inlineStr">
+      <c r="B29" s="125" t="inlineStr">
         <is>
           <t>Category (weight)</t>
         </is>
@@ -5468,7 +5470,7 @@
           <t>Team avg (0-5)</t>
         </is>
       </c>
-      <c r="D29" s="116" t="inlineStr">
+      <c r="D29" s="125" t="inlineStr">
         <is>
           <t>What the journey shows</t>
         </is>
@@ -5605,17 +5607,17 @@
       <c r="D39" s="68" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="116" t="inlineStr">
+      <c r="B40" s="125" t="inlineStr">
         <is>
           <t>Opportunity (category)</t>
         </is>
       </c>
-      <c r="C40" s="116" t="inlineStr">
+      <c r="C40" s="125" t="inlineStr">
         <is>
           <t>Evidence across touches (why it's a TEAM issue, not one agent)</t>
         </is>
       </c>
-      <c r="D40" s="116" t="inlineStr">
+      <c r="D40" s="125" t="inlineStr">
         <is>
           <t>Team action &amp; suggested owner</t>
         </is>
@@ -5758,7 +5760,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="116" t="inlineStr">
+      <c r="B50" s="125" t="inlineStr">
         <is>
           <t>6 · HOW TO RUN A TEAM REVIEW FOR YOUR OWN JOURNEYS (~30 min once touches are scored)</t>
         </is>
@@ -5859,6 +5861,8 @@
           <t>7 · CONTRIBUTION TYPE &amp; HANDOFF QUALITY — LIVE PER-TOUCH BREAKDOWN</t>
         </is>
       </c>
+      <c r="C60" s="67" t="n"/>
+      <c r="D60" s="68" t="n"/>
     </row>
     <row r="61" ht="32" customHeight="1">
       <c r="B61" s="52" t="inlineStr">
@@ -5866,12 +5870,16 @@
           <t>Pulled live from the Case Tracker (columns O &amp; P). Use this to judge the Continuity &amp; Handoffs component above — it shows WHERE the chain held and WHERE it broke, touch by touch, instead of one averaged number.</t>
         </is>
       </c>
+      <c r="C61" s="67" t="n"/>
+      <c r="D61" s="68" t="n"/>
     </row>
     <row r="62" ht="34" customHeight="1">
       <c r="B62" s="128">
-        <f>"Contribution mix across 13 touches:  "&amp;COUNTIF('Case Tracker'!O5:O17,"Resolver")&amp;" Resolver · "&amp;COUNTIF('Case Tracker'!O5:O17,"Progress Builder")&amp;" Progress Builder · "&amp;COUNTIF('Case Tracker'!O5:O17,"Maintainer")&amp;" Maintainer · "&amp;COUNTIF('Case Tracker'!O5:O17,"Breaker")&amp;" Breaker.   Average Handoff Quality (touches 1-12): "&amp;TEXT(AVERAGE('Case Tracker'!P5:P16),"0.0")&amp;" / 5"</f>
-        <v/>
-      </c>
+        <f>"Contribution mix across 13 touches:  "&amp;COUNTIF('Case Tracker'!O5:O17,"Resolver")&amp;" Resolver · "&amp;COUNTIF('Case Tracker'!O5:O17,"Progress Builder")&amp;" Progress Builder · "&amp;COUNTIF('Case Tracker'!O5:O17,"Maintainer")&amp;" Maintainer · "&amp;COUNTIF('Case Tracker'!O5:O17,"Regression Contributor")&amp;" Regression Contributor.   Average Handoff Quality (touches 1-12): "&amp;TEXT(AVERAGE('Case Tracker'!P5:P16),"0.0")&amp;" / 5"</f>
+        <v/>
+      </c>
+      <c r="C62" s="67" t="n"/>
+      <c r="D62" s="68" t="n"/>
     </row>
     <row r="63" ht="24" customHeight="1">
       <c r="B63" s="129" t="inlineStr">
@@ -6075,9 +6083,11 @@
     <row r="77" ht="40" customHeight="1">
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>Reading this table: a long run of Breaker / low Handoff Quality rows is a process problem (closure discipline, callback management), not an individual one — see Team Opportunities above. A single Breaker surrounded by Resolvers/Progress Builders points at one agent or one moment, and belongs in that agent's individual coaching instead.</t>
-        </is>
-      </c>
+          <t>Reading this table: a long run of Regression Contributor / low Handoff Quality rows is a process problem (closure discipline, callback management), not an individual one — see Team Opportunities above. A single Regression Contributor surrounded by Resolvers/Progress Builders points at one agent or one moment, and belongs in that agent's individual coaching instead.</t>
+        </is>
+      </c>
+      <c r="C77" s="70" t="n"/>
+      <c r="D77" s="69" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="29">
@@ -6154,7 +6164,7 @@
       <formula>"Maintainer"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="12" operator="equal" dxfId="2">
-      <formula>"Breaker"</formula>
+      <formula>"Regression Contributor"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D64:D76">
@@ -6214,7 +6224,7 @@
       <c r="F2" s="68" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="116" t="inlineStr">
+      <c r="B4" s="125" t="inlineStr">
         <is>
           <t>1 · CASE INFORMATION</t>
         </is>
@@ -6450,7 +6460,7 @@
       <c r="F16" s="68" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="116" t="inlineStr">
+      <c r="B17" s="125" t="inlineStr">
         <is>
           <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
@@ -6646,7 +6656,7 @@
       <c r="F28" s="69" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="116" t="inlineStr">
+      <c r="B30" s="125" t="inlineStr">
         <is>
           <t>2. TECHNICAL ACCURACY</t>
         </is>
@@ -6880,7 +6890,7 @@
       <c r="F43" s="69" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="B45" s="116" t="inlineStr">
+      <c r="B45" s="125" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
@@ -7133,7 +7143,7 @@
       <c r="F59" s="69" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="B61" s="116" t="inlineStr">
+      <c r="B61" s="125" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
@@ -7386,7 +7396,7 @@
       <c r="F75" s="69" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="B77" s="116" t="inlineStr">
+      <c r="B77" s="125" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
@@ -7582,7 +7592,7 @@
       <c r="F88" s="69" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="B90" s="116" t="inlineStr">
+      <c r="B90" s="125" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
@@ -7797,7 +7807,7 @@
       <c r="F102" s="69" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="B104" s="116" t="inlineStr">
+      <c r="B104" s="125" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
@@ -8085,7 +8095,7 @@
         <f>IF(D121="","",(D121/5)*C121)</f>
         <v/>
       </c>
-      <c r="F121" s="82">
+      <c r="F121" s="132">
         <f>IF(D121="","",IF(D121&gt;=4,"Strong",IF(D121=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8107,7 +8117,7 @@
         <f>IF(D122="","",(D122/5)*C122)</f>
         <v/>
       </c>
-      <c r="F122" s="77">
+      <c r="F122" s="131">
         <f>IF(D122="","",IF(D122&gt;=4,"Strong",IF(D122=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8129,7 +8139,7 @@
         <f>IF(D123="","",(D123/5)*C123)</f>
         <v/>
       </c>
-      <c r="F123" s="82">
+      <c r="F123" s="132">
         <f>IF(D123="","",IF(D123&gt;=4,"Strong",IF(D123=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8151,7 +8161,7 @@
         <f>IF(D124="","",(D124/5)*C124)</f>
         <v/>
       </c>
-      <c r="F124" s="77">
+      <c r="F124" s="131">
         <f>IF(D124="","",IF(D124&gt;=4,"Strong",IF(D124=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8173,7 +8183,7 @@
         <f>IF(D125="","",(D125/5)*C125)</f>
         <v/>
       </c>
-      <c r="F125" s="82">
+      <c r="F125" s="132">
         <f>IF(D125="","",IF(D125&gt;=4,"Strong",IF(D125=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8195,7 +8205,7 @@
         <f>IF(D126="","",(D126/5)*C126)</f>
         <v/>
       </c>
-      <c r="F126" s="77">
+      <c r="F126" s="131">
         <f>IF(D126="","",IF(D126&gt;=4,"Strong",IF(D126=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8217,7 +8227,7 @@
         <f>IF(D127="","",(D127/5)*C127)</f>
         <v/>
       </c>
-      <c r="F127" s="82">
+      <c r="F127" s="132">
         <f>IF(D127="","",IF(D127&gt;=4,"Strong",IF(D127=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
@@ -8243,7 +8253,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="116" t="inlineStr">
+      <c r="B130" s="125" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
@@ -8299,7 +8309,7 @@
       <c r="F133" s="69" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="116" t="inlineStr">
+      <c r="B135" s="125" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
@@ -8358,7 +8368,7 @@
       <c r="F139" s="68" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="116" t="inlineStr">
+      <c r="B140" s="125" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
@@ -8368,7 +8378,7 @@
           <t>Present?</t>
         </is>
       </c>
-      <c r="D140" s="116" t="inlineStr">
+      <c r="D140" s="125" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
@@ -8579,7 +8589,7 @@
       <c r="F154" s="68" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="116" t="inlineStr">
+      <c r="B155" s="125" t="inlineStr">
         <is>
           <t>WHAT WENT WELL — behaviors to repeat</t>
         </is>
@@ -8635,7 +8645,7 @@
       <c r="F158" s="69" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="116" t="inlineStr">
+      <c r="B159" s="125" t="inlineStr">
         <is>
           <t>IMPROVEMENT OPPORTUNITIES — behaviors to improve</t>
         </is>
@@ -8691,7 +8701,7 @@
       <c r="F162" s="69" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="116" t="inlineStr">
+      <c r="B163" s="125" t="inlineStr">
         <is>
           <t>COACHING RECOMMENDATION — specific actions the agent should apply going forward</t>
         </is>
@@ -8713,7 +8723,7 @@
       <c r="F164" s="69" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="116" t="inlineStr">
+      <c r="B165" s="125" t="inlineStr">
         <is>
           <t>ORGANIZATIONAL INSIGHTS — training / process / KB / chatbot / tooling / product gaps discovered</t>
         </is>
@@ -8735,7 +8745,7 @@
       <c r="F166" s="69" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="116" t="inlineStr">
+      <c r="B167" s="125" t="inlineStr">
         <is>
           <t>MULTI-TOUCH / JOURNEY NOTES — handoff quality received &amp; passed, continuity, where the chain stands</t>
         </is>
@@ -8757,7 +8767,7 @@
       <c r="F168" s="69" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="116" t="inlineStr">
+      <c r="B169" s="125" t="inlineStr">
         <is>
           <t>FINAL QA ASSESSMENT — customer outcome, support quality, and coaching value</t>
         </is>
@@ -9188,7 +9198,7 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -9383,7 +9393,7 @@
         <f>IF((COUNT(E5)+COUNT(F5)+COUNT(G5)+COUNT(H5)+COUNT(I5)+COUNT(J5)+COUNT(K5))=0,"",IFERROR(E5/5*0.3,0)+IFERROR(F5/5*0.2,0)+IFERROR(G5/5*0.15,0)+IFERROR(H5/5*0.15,0)+IFERROR(I5/5*0.1,0)+IFERROR(J5/5*0.05,0)+IFERROR(K5/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M5" s="82">
+      <c r="M5" s="132">
         <f>IF(L5="","",IF(L5&gt;=0.85,"Meets/Exceeds",IF(L5&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9445,7 +9455,7 @@
         <f>IF((COUNT(E6)+COUNT(F6)+COUNT(G6)+COUNT(H6)+COUNT(I6)+COUNT(J6)+COUNT(K6))=0,"",IFERROR(E6/5*0.3,0)+IFERROR(F6/5*0.2,0)+IFERROR(G6/5*0.15,0)+IFERROR(H6/5*0.15,0)+IFERROR(I6/5*0.1,0)+IFERROR(J6/5*0.05,0)+IFERROR(K6/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M6" s="77">
+      <c r="M6" s="131">
         <f>IF(L6="","",IF(L6&gt;=0.85,"Meets/Exceeds",IF(L6&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9456,7 +9466,7 @@
       </c>
       <c r="O6" s="131" t="inlineStr">
         <is>
-          <t>Breaker</t>
+          <t>Regression Contributor</t>
         </is>
       </c>
       <c r="P6" s="131" t="n">
@@ -9507,7 +9517,7 @@
         <f>IF((COUNT(E7)+COUNT(F7)+COUNT(G7)+COUNT(H7)+COUNT(I7)+COUNT(J7)+COUNT(K7))=0,"",IFERROR(E7/5*0.3,0)+IFERROR(F7/5*0.2,0)+IFERROR(G7/5*0.15,0)+IFERROR(H7/5*0.15,0)+IFERROR(I7/5*0.1,0)+IFERROR(J7/5*0.05,0)+IFERROR(K7/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M7" s="82">
+      <c r="M7" s="132">
         <f>IF(L7="","",IF(L7&gt;=0.85,"Meets/Exceeds",IF(L7&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9569,7 +9579,7 @@
         <f>IF((COUNT(E8)+COUNT(F8)+COUNT(G8)+COUNT(H8)+COUNT(I8)+COUNT(J8)+COUNT(K8))=0,"",IFERROR(E8/5*0.3,0)+IFERROR(F8/5*0.2,0)+IFERROR(G8/5*0.15,0)+IFERROR(H8/5*0.15,0)+IFERROR(I8/5*0.1,0)+IFERROR(J8/5*0.05,0)+IFERROR(K8/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M8" s="77">
+      <c r="M8" s="131">
         <f>IF(L8="","",IF(L8&gt;=0.85,"Meets/Exceeds",IF(L8&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9631,7 +9641,7 @@
         <f>IF((COUNT(E9)+COUNT(F9)+COUNT(G9)+COUNT(H9)+COUNT(I9)+COUNT(J9)+COUNT(K9))=0,"",IFERROR(E9/5*0.3,0)+IFERROR(F9/5*0.2,0)+IFERROR(G9/5*0.15,0)+IFERROR(H9/5*0.15,0)+IFERROR(I9/5*0.1,0)+IFERROR(J9/5*0.05,0)+IFERROR(K9/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M9" s="82">
+      <c r="M9" s="132">
         <f>IF(L9="","",IF(L9&gt;=0.85,"Meets/Exceeds",IF(L9&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9693,7 +9703,7 @@
         <f>IF((COUNT(E10)+COUNT(F10)+COUNT(G10)+COUNT(H10)+COUNT(I10)+COUNT(J10)+COUNT(K10))=0,"",IFERROR(E10/5*0.3,0)+IFERROR(F10/5*0.2,0)+IFERROR(G10/5*0.15,0)+IFERROR(H10/5*0.15,0)+IFERROR(I10/5*0.1,0)+IFERROR(J10/5*0.05,0)+IFERROR(K10/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M10" s="77">
+      <c r="M10" s="131">
         <f>IF(L10="","",IF(L10&gt;=0.85,"Meets/Exceeds",IF(L10&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9755,7 +9765,7 @@
         <f>IF((COUNT(E11)+COUNT(F11)+COUNT(G11)+COUNT(H11)+COUNT(I11)+COUNT(J11)+COUNT(K11))=0,"",IFERROR(E11/5*0.3,0)+IFERROR(F11/5*0.2,0)+IFERROR(G11/5*0.15,0)+IFERROR(H11/5*0.15,0)+IFERROR(I11/5*0.1,0)+IFERROR(J11/5*0.05,0)+IFERROR(K11/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M11" s="82">
+      <c r="M11" s="132">
         <f>IF(L11="","",IF(L11&gt;=0.85,"Meets/Exceeds",IF(L11&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9766,7 +9776,7 @@
       </c>
       <c r="O11" s="132" t="inlineStr">
         <is>
-          <t>Breaker</t>
+          <t>Regression Contributor</t>
         </is>
       </c>
       <c r="P11" s="132" t="n">
@@ -9817,7 +9827,7 @@
         <f>IF((COUNT(E12)+COUNT(F12)+COUNT(G12)+COUNT(H12)+COUNT(I12)+COUNT(J12)+COUNT(K12))=0,"",IFERROR(E12/5*0.3,0)+IFERROR(F12/5*0.2,0)+IFERROR(G12/5*0.15,0)+IFERROR(H12/5*0.15,0)+IFERROR(I12/5*0.1,0)+IFERROR(J12/5*0.05,0)+IFERROR(K12/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M12" s="77">
+      <c r="M12" s="131">
         <f>IF(L12="","",IF(L12&gt;=0.85,"Meets/Exceeds",IF(L12&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9828,7 +9838,7 @@
       </c>
       <c r="O12" s="131" t="inlineStr">
         <is>
-          <t>Breaker</t>
+          <t>Regression Contributor</t>
         </is>
       </c>
       <c r="P12" s="131" t="n">
@@ -9879,7 +9889,7 @@
         <f>IF((COUNT(E13)+COUNT(F13)+COUNT(G13)+COUNT(H13)+COUNT(I13)+COUNT(J13)+COUNT(K13))=0,"",IFERROR(E13/5*0.3,0)+IFERROR(F13/5*0.2,0)+IFERROR(G13/5*0.15,0)+IFERROR(H13/5*0.15,0)+IFERROR(I13/5*0.1,0)+IFERROR(J13/5*0.05,0)+IFERROR(K13/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M13" s="82">
+      <c r="M13" s="132">
         <f>IF(L13="","",IF(L13&gt;=0.85,"Meets/Exceeds",IF(L13&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -9941,7 +9951,7 @@
         <f>IF((COUNT(E14)+COUNT(F14)+COUNT(G14)+COUNT(H14)+COUNT(I14)+COUNT(J14)+COUNT(K14))=0,"",IFERROR(E14/5*0.3,0)+IFERROR(F14/5*0.2,0)+IFERROR(G14/5*0.15,0)+IFERROR(H14/5*0.15,0)+IFERROR(I14/5*0.1,0)+IFERROR(J14/5*0.05,0)+IFERROR(K14/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M14" s="77">
+      <c r="M14" s="131">
         <f>IF(L14="","",IF(L14&gt;=0.85,"Meets/Exceeds",IF(L14&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10003,7 +10013,7 @@
         <f>IF((COUNT(E15)+COUNT(F15)+COUNT(G15)+COUNT(H15)+COUNT(I15)+COUNT(J15)+COUNT(K15))=0,"",IFERROR(E15/5*0.3,0)+IFERROR(F15/5*0.2,0)+IFERROR(G15/5*0.15,0)+IFERROR(H15/5*0.15,0)+IFERROR(I15/5*0.1,0)+IFERROR(J15/5*0.05,0)+IFERROR(K15/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M15" s="82">
+      <c r="M15" s="132">
         <f>IF(L15="","",IF(L15&gt;=0.85,"Meets/Exceeds",IF(L15&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10065,7 +10075,7 @@
         <f>IF((COUNT(E16)+COUNT(F16)+COUNT(G16)+COUNT(H16)+COUNT(I16)+COUNT(J16)+COUNT(K16))=0,"",IFERROR(E16/5*0.3,0)+IFERROR(F16/5*0.2,0)+IFERROR(G16/5*0.15,0)+IFERROR(H16/5*0.15,0)+IFERROR(I16/5*0.1,0)+IFERROR(J16/5*0.05,0)+IFERROR(K16/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M16" s="77">
+      <c r="M16" s="131">
         <f>IF(L16="","",IF(L16&gt;=0.85,"Meets/Exceeds",IF(L16&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10127,7 +10137,7 @@
         <f>IF((COUNT(E17)+COUNT(F17)+COUNT(G17)+COUNT(H17)+COUNT(I17)+COUNT(J17)+COUNT(K17))=0,"",IFERROR(E17/5*0.3,0)+IFERROR(F17/5*0.2,0)+IFERROR(G17/5*0.15,0)+IFERROR(H17/5*0.15,0)+IFERROR(I17/5*0.1,0)+IFERROR(J17/5*0.05,0)+IFERROR(K17/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M17" s="82">
+      <c r="M17" s="132">
         <f>IF(L17="","",IF(L17&gt;=0.85,"Meets/Exceeds",IF(L17&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10163,7 +10173,7 @@
         <f>IF((COUNT(E18)+COUNT(F18)+COUNT(G18)+COUNT(H18)+COUNT(I18)+COUNT(J18)+COUNT(K18))=0,"",IFERROR(E18/5*0.3,0)+IFERROR(F18/5*0.2,0)+IFERROR(G18/5*0.15,0)+IFERROR(H18/5*0.15,0)+IFERROR(I18/5*0.1,0)+IFERROR(J18/5*0.05,0)+IFERROR(K18/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M18" s="77">
+      <c r="M18" s="131">
         <f>IF(L18="","",IF(L18&gt;=0.85,"Meets/Exceeds",IF(L18&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10187,7 +10197,7 @@
         <f>IF((COUNT(E19)+COUNT(F19)+COUNT(G19)+COUNT(H19)+COUNT(I19)+COUNT(J19)+COUNT(K19))=0,"",IFERROR(E19/5*0.3,0)+IFERROR(F19/5*0.2,0)+IFERROR(G19/5*0.15,0)+IFERROR(H19/5*0.15,0)+IFERROR(I19/5*0.1,0)+IFERROR(J19/5*0.05,0)+IFERROR(K19/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M19" s="82">
+      <c r="M19" s="132">
         <f>IF(L19="","",IF(L19&gt;=0.85,"Meets/Exceeds",IF(L19&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10211,7 +10221,7 @@
         <f>IF((COUNT(E20)+COUNT(F20)+COUNT(G20)+COUNT(H20)+COUNT(I20)+COUNT(J20)+COUNT(K20))=0,"",IFERROR(E20/5*0.3,0)+IFERROR(F20/5*0.2,0)+IFERROR(G20/5*0.15,0)+IFERROR(H20/5*0.15,0)+IFERROR(I20/5*0.1,0)+IFERROR(J20/5*0.05,0)+IFERROR(K20/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M20" s="77">
+      <c r="M20" s="131">
         <f>IF(L20="","",IF(L20&gt;=0.85,"Meets/Exceeds",IF(L20&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10235,7 +10245,7 @@
         <f>IF((COUNT(E21)+COUNT(F21)+COUNT(G21)+COUNT(H21)+COUNT(I21)+COUNT(J21)+COUNT(K21))=0,"",IFERROR(E21/5*0.3,0)+IFERROR(F21/5*0.2,0)+IFERROR(G21/5*0.15,0)+IFERROR(H21/5*0.15,0)+IFERROR(I21/5*0.1,0)+IFERROR(J21/5*0.05,0)+IFERROR(K21/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M21" s="82">
+      <c r="M21" s="132">
         <f>IF(L21="","",IF(L21&gt;=0.85,"Meets/Exceeds",IF(L21&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10259,7 +10269,7 @@
         <f>IF((COUNT(E22)+COUNT(F22)+COUNT(G22)+COUNT(H22)+COUNT(I22)+COUNT(J22)+COUNT(K22))=0,"",IFERROR(E22/5*0.3,0)+IFERROR(F22/5*0.2,0)+IFERROR(G22/5*0.15,0)+IFERROR(H22/5*0.15,0)+IFERROR(I22/5*0.1,0)+IFERROR(J22/5*0.05,0)+IFERROR(K22/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M22" s="77">
+      <c r="M22" s="131">
         <f>IF(L22="","",IF(L22&gt;=0.85,"Meets/Exceeds",IF(L22&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10283,7 +10293,7 @@
         <f>IF((COUNT(E23)+COUNT(F23)+COUNT(G23)+COUNT(H23)+COUNT(I23)+COUNT(J23)+COUNT(K23))=0,"",IFERROR(E23/5*0.3,0)+IFERROR(F23/5*0.2,0)+IFERROR(G23/5*0.15,0)+IFERROR(H23/5*0.15,0)+IFERROR(I23/5*0.1,0)+IFERROR(J23/5*0.05,0)+IFERROR(K23/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M23" s="82">
+      <c r="M23" s="132">
         <f>IF(L23="","",IF(L23&gt;=0.85,"Meets/Exceeds",IF(L23&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10307,7 +10317,7 @@
         <f>IF((COUNT(E24)+COUNT(F24)+COUNT(G24)+COUNT(H24)+COUNT(I24)+COUNT(J24)+COUNT(K24))=0,"",IFERROR(E24/5*0.3,0)+IFERROR(F24/5*0.2,0)+IFERROR(G24/5*0.15,0)+IFERROR(H24/5*0.15,0)+IFERROR(I24/5*0.1,0)+IFERROR(J24/5*0.05,0)+IFERROR(K24/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M24" s="77">
+      <c r="M24" s="131">
         <f>IF(L24="","",IF(L24&gt;=0.85,"Meets/Exceeds",IF(L24&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10331,7 +10341,7 @@
         <f>IF((COUNT(E25)+COUNT(F25)+COUNT(G25)+COUNT(H25)+COUNT(I25)+COUNT(J25)+COUNT(K25))=0,"",IFERROR(E25/5*0.3,0)+IFERROR(F25/5*0.2,0)+IFERROR(G25/5*0.15,0)+IFERROR(H25/5*0.15,0)+IFERROR(I25/5*0.1,0)+IFERROR(J25/5*0.05,0)+IFERROR(K25/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M25" s="82">
+      <c r="M25" s="132">
         <f>IF(L25="","",IF(L25&gt;=0.85,"Meets/Exceeds",IF(L25&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10355,7 +10365,7 @@
         <f>IF((COUNT(E26)+COUNT(F26)+COUNT(G26)+COUNT(H26)+COUNT(I26)+COUNT(J26)+COUNT(K26))=0,"",IFERROR(E26/5*0.3,0)+IFERROR(F26/5*0.2,0)+IFERROR(G26/5*0.15,0)+IFERROR(H26/5*0.15,0)+IFERROR(I26/5*0.1,0)+IFERROR(J26/5*0.05,0)+IFERROR(K26/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M26" s="77">
+      <c r="M26" s="131">
         <f>IF(L26="","",IF(L26&gt;=0.85,"Meets/Exceeds",IF(L26&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10379,7 +10389,7 @@
         <f>IF((COUNT(E27)+COUNT(F27)+COUNT(G27)+COUNT(H27)+COUNT(I27)+COUNT(J27)+COUNT(K27))=0,"",IFERROR(E27/5*0.3,0)+IFERROR(F27/5*0.2,0)+IFERROR(G27/5*0.15,0)+IFERROR(H27/5*0.15,0)+IFERROR(I27/5*0.1,0)+IFERROR(J27/5*0.05,0)+IFERROR(K27/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M27" s="82">
+      <c r="M27" s="132">
         <f>IF(L27="","",IF(L27&gt;=0.85,"Meets/Exceeds",IF(L27&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10403,7 +10413,7 @@
         <f>IF((COUNT(E28)+COUNT(F28)+COUNT(G28)+COUNT(H28)+COUNT(I28)+COUNT(J28)+COUNT(K28))=0,"",IFERROR(E28/5*0.3,0)+IFERROR(F28/5*0.2,0)+IFERROR(G28/5*0.15,0)+IFERROR(H28/5*0.15,0)+IFERROR(I28/5*0.1,0)+IFERROR(J28/5*0.05,0)+IFERROR(K28/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M28" s="77">
+      <c r="M28" s="131">
         <f>IF(L28="","",IF(L28&gt;=0.85,"Meets/Exceeds",IF(L28&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10427,7 +10437,7 @@
         <f>IF((COUNT(E29)+COUNT(F29)+COUNT(G29)+COUNT(H29)+COUNT(I29)+COUNT(J29)+COUNT(K29))=0,"",IFERROR(E29/5*0.3,0)+IFERROR(F29/5*0.2,0)+IFERROR(G29/5*0.15,0)+IFERROR(H29/5*0.15,0)+IFERROR(I29/5*0.1,0)+IFERROR(J29/5*0.05,0)+IFERROR(K29/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M29" s="82">
+      <c r="M29" s="132">
         <f>IF(L29="","",IF(L29&gt;=0.85,"Meets/Exceeds",IF(L29&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10451,7 +10461,7 @@
         <f>IF((COUNT(E30)+COUNT(F30)+COUNT(G30)+COUNT(H30)+COUNT(I30)+COUNT(J30)+COUNT(K30))=0,"",IFERROR(E30/5*0.3,0)+IFERROR(F30/5*0.2,0)+IFERROR(G30/5*0.15,0)+IFERROR(H30/5*0.15,0)+IFERROR(I30/5*0.1,0)+IFERROR(J30/5*0.05,0)+IFERROR(K30/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M30" s="77">
+      <c r="M30" s="131">
         <f>IF(L30="","",IF(L30&gt;=0.85,"Meets/Exceeds",IF(L30&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10475,7 +10485,7 @@
         <f>IF((COUNT(E31)+COUNT(F31)+COUNT(G31)+COUNT(H31)+COUNT(I31)+COUNT(J31)+COUNT(K31))=0,"",IFERROR(E31/5*0.3,0)+IFERROR(F31/5*0.2,0)+IFERROR(G31/5*0.15,0)+IFERROR(H31/5*0.15,0)+IFERROR(I31/5*0.1,0)+IFERROR(J31/5*0.05,0)+IFERROR(K31/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M31" s="82">
+      <c r="M31" s="132">
         <f>IF(L31="","",IF(L31&gt;=0.85,"Meets/Exceeds",IF(L31&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10499,7 +10509,7 @@
         <f>IF((COUNT(E32)+COUNT(F32)+COUNT(G32)+COUNT(H32)+COUNT(I32)+COUNT(J32)+COUNT(K32))=0,"",IFERROR(E32/5*0.3,0)+IFERROR(F32/5*0.2,0)+IFERROR(G32/5*0.15,0)+IFERROR(H32/5*0.15,0)+IFERROR(I32/5*0.1,0)+IFERROR(J32/5*0.05,0)+IFERROR(K32/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M32" s="77">
+      <c r="M32" s="131">
         <f>IF(L32="","",IF(L32&gt;=0.85,"Meets/Exceeds",IF(L32&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10523,7 +10533,7 @@
         <f>IF((COUNT(E33)+COUNT(F33)+COUNT(G33)+COUNT(H33)+COUNT(I33)+COUNT(J33)+COUNT(K33))=0,"",IFERROR(E33/5*0.3,0)+IFERROR(F33/5*0.2,0)+IFERROR(G33/5*0.15,0)+IFERROR(H33/5*0.15,0)+IFERROR(I33/5*0.1,0)+IFERROR(J33/5*0.05,0)+IFERROR(K33/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M33" s="82">
+      <c r="M33" s="132">
         <f>IF(L33="","",IF(L33&gt;=0.85,"Meets/Exceeds",IF(L33&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10547,7 +10557,7 @@
         <f>IF((COUNT(E34)+COUNT(F34)+COUNT(G34)+COUNT(H34)+COUNT(I34)+COUNT(J34)+COUNT(K34))=0,"",IFERROR(E34/5*0.3,0)+IFERROR(F34/5*0.2,0)+IFERROR(G34/5*0.15,0)+IFERROR(H34/5*0.15,0)+IFERROR(I34/5*0.1,0)+IFERROR(J34/5*0.05,0)+IFERROR(K34/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M34" s="77">
+      <c r="M34" s="131">
         <f>IF(L34="","",IF(L34&gt;=0.85,"Meets/Exceeds",IF(L34&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10571,7 +10581,7 @@
         <f>IF((COUNT(E35)+COUNT(F35)+COUNT(G35)+COUNT(H35)+COUNT(I35)+COUNT(J35)+COUNT(K35))=0,"",IFERROR(E35/5*0.3,0)+IFERROR(F35/5*0.2,0)+IFERROR(G35/5*0.15,0)+IFERROR(H35/5*0.15,0)+IFERROR(I35/5*0.1,0)+IFERROR(J35/5*0.05,0)+IFERROR(K35/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M35" s="82">
+      <c r="M35" s="132">
         <f>IF(L35="","",IF(L35&gt;=0.85,"Meets/Exceeds",IF(L35&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10595,7 +10605,7 @@
         <f>IF((COUNT(E36)+COUNT(F36)+COUNT(G36)+COUNT(H36)+COUNT(I36)+COUNT(J36)+COUNT(K36))=0,"",IFERROR(E36/5*0.3,0)+IFERROR(F36/5*0.2,0)+IFERROR(G36/5*0.15,0)+IFERROR(H36/5*0.15,0)+IFERROR(I36/5*0.1,0)+IFERROR(J36/5*0.05,0)+IFERROR(K36/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M36" s="77">
+      <c r="M36" s="131">
         <f>IF(L36="","",IF(L36&gt;=0.85,"Meets/Exceeds",IF(L36&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10619,7 +10629,7 @@
         <f>IF((COUNT(E37)+COUNT(F37)+COUNT(G37)+COUNT(H37)+COUNT(I37)+COUNT(J37)+COUNT(K37))=0,"",IFERROR(E37/5*0.3,0)+IFERROR(F37/5*0.2,0)+IFERROR(G37/5*0.15,0)+IFERROR(H37/5*0.15,0)+IFERROR(I37/5*0.1,0)+IFERROR(J37/5*0.05,0)+IFERROR(K37/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M37" s="82">
+      <c r="M37" s="132">
         <f>IF(L37="","",IF(L37&gt;=0.85,"Meets/Exceeds",IF(L37&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10643,7 +10653,7 @@
         <f>IF((COUNT(E38)+COUNT(F38)+COUNT(G38)+COUNT(H38)+COUNT(I38)+COUNT(J38)+COUNT(K38))=0,"",IFERROR(E38/5*0.3,0)+IFERROR(F38/5*0.2,0)+IFERROR(G38/5*0.15,0)+IFERROR(H38/5*0.15,0)+IFERROR(I38/5*0.1,0)+IFERROR(J38/5*0.05,0)+IFERROR(K38/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M38" s="77">
+      <c r="M38" s="131">
         <f>IF(L38="","",IF(L38&gt;=0.85,"Meets/Exceeds",IF(L38&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10667,7 +10677,7 @@
         <f>IF((COUNT(E39)+COUNT(F39)+COUNT(G39)+COUNT(H39)+COUNT(I39)+COUNT(J39)+COUNT(K39))=0,"",IFERROR(E39/5*0.3,0)+IFERROR(F39/5*0.2,0)+IFERROR(G39/5*0.15,0)+IFERROR(H39/5*0.15,0)+IFERROR(I39/5*0.1,0)+IFERROR(J39/5*0.05,0)+IFERROR(K39/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M39" s="82">
+      <c r="M39" s="132">
         <f>IF(L39="","",IF(L39&gt;=0.85,"Meets/Exceeds",IF(L39&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10691,7 +10701,7 @@
         <f>IF((COUNT(E40)+COUNT(F40)+COUNT(G40)+COUNT(H40)+COUNT(I40)+COUNT(J40)+COUNT(K40))=0,"",IFERROR(E40/5*0.3,0)+IFERROR(F40/5*0.2,0)+IFERROR(G40/5*0.15,0)+IFERROR(H40/5*0.15,0)+IFERROR(I40/5*0.1,0)+IFERROR(J40/5*0.05,0)+IFERROR(K40/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M40" s="77">
+      <c r="M40" s="131">
         <f>IF(L40="","",IF(L40&gt;=0.85,"Meets/Exceeds",IF(L40&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10715,7 +10725,7 @@
         <f>IF((COUNT(E41)+COUNT(F41)+COUNT(G41)+COUNT(H41)+COUNT(I41)+COUNT(J41)+COUNT(K41))=0,"",IFERROR(E41/5*0.3,0)+IFERROR(F41/5*0.2,0)+IFERROR(G41/5*0.15,0)+IFERROR(H41/5*0.15,0)+IFERROR(I41/5*0.1,0)+IFERROR(J41/5*0.05,0)+IFERROR(K41/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M41" s="82">
+      <c r="M41" s="132">
         <f>IF(L41="","",IF(L41&gt;=0.85,"Meets/Exceeds",IF(L41&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10739,7 +10749,7 @@
         <f>IF((COUNT(E42)+COUNT(F42)+COUNT(G42)+COUNT(H42)+COUNT(I42)+COUNT(J42)+COUNT(K42))=0,"",IFERROR(E42/5*0.3,0)+IFERROR(F42/5*0.2,0)+IFERROR(G42/5*0.15,0)+IFERROR(H42/5*0.15,0)+IFERROR(I42/5*0.1,0)+IFERROR(J42/5*0.05,0)+IFERROR(K42/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M42" s="77">
+      <c r="M42" s="131">
         <f>IF(L42="","",IF(L42&gt;=0.85,"Meets/Exceeds",IF(L42&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10763,7 +10773,7 @@
         <f>IF((COUNT(E43)+COUNT(F43)+COUNT(G43)+COUNT(H43)+COUNT(I43)+COUNT(J43)+COUNT(K43))=0,"",IFERROR(E43/5*0.3,0)+IFERROR(F43/5*0.2,0)+IFERROR(G43/5*0.15,0)+IFERROR(H43/5*0.15,0)+IFERROR(I43/5*0.1,0)+IFERROR(J43/5*0.05,0)+IFERROR(K43/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M43" s="82">
+      <c r="M43" s="132">
         <f>IF(L43="","",IF(L43&gt;=0.85,"Meets/Exceeds",IF(L43&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10787,7 +10797,7 @@
         <f>IF((COUNT(E44)+COUNT(F44)+COUNT(G44)+COUNT(H44)+COUNT(I44)+COUNT(J44)+COUNT(K44))=0,"",IFERROR(E44/5*0.3,0)+IFERROR(F44/5*0.2,0)+IFERROR(G44/5*0.15,0)+IFERROR(H44/5*0.15,0)+IFERROR(I44/5*0.1,0)+IFERROR(J44/5*0.05,0)+IFERROR(K44/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M44" s="77">
+      <c r="M44" s="131">
         <f>IF(L44="","",IF(L44&gt;=0.85,"Meets/Exceeds",IF(L44&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10811,7 +10821,7 @@
         <f>IF((COUNT(E45)+COUNT(F45)+COUNT(G45)+COUNT(H45)+COUNT(I45)+COUNT(J45)+COUNT(K45))=0,"",IFERROR(E45/5*0.3,0)+IFERROR(F45/5*0.2,0)+IFERROR(G45/5*0.15,0)+IFERROR(H45/5*0.15,0)+IFERROR(I45/5*0.1,0)+IFERROR(J45/5*0.05,0)+IFERROR(K45/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M45" s="82">
+      <c r="M45" s="132">
         <f>IF(L45="","",IF(L45&gt;=0.85,"Meets/Exceeds",IF(L45&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10835,7 +10845,7 @@
         <f>IF((COUNT(E46)+COUNT(F46)+COUNT(G46)+COUNT(H46)+COUNT(I46)+COUNT(J46)+COUNT(K46))=0,"",IFERROR(E46/5*0.3,0)+IFERROR(F46/5*0.2,0)+IFERROR(G46/5*0.15,0)+IFERROR(H46/5*0.15,0)+IFERROR(I46/5*0.1,0)+IFERROR(J46/5*0.05,0)+IFERROR(K46/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M46" s="77">
+      <c r="M46" s="131">
         <f>IF(L46="","",IF(L46&gt;=0.85,"Meets/Exceeds",IF(L46&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10859,7 +10869,7 @@
         <f>IF((COUNT(E47)+COUNT(F47)+COUNT(G47)+COUNT(H47)+COUNT(I47)+COUNT(J47)+COUNT(K47))=0,"",IFERROR(E47/5*0.3,0)+IFERROR(F47/5*0.2,0)+IFERROR(G47/5*0.15,0)+IFERROR(H47/5*0.15,0)+IFERROR(I47/5*0.1,0)+IFERROR(J47/5*0.05,0)+IFERROR(K47/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M47" s="82">
+      <c r="M47" s="132">
         <f>IF(L47="","",IF(L47&gt;=0.85,"Meets/Exceeds",IF(L47&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10883,7 +10893,7 @@
         <f>IF((COUNT(E48)+COUNT(F48)+COUNT(G48)+COUNT(H48)+COUNT(I48)+COUNT(J48)+COUNT(K48))=0,"",IFERROR(E48/5*0.3,0)+IFERROR(F48/5*0.2,0)+IFERROR(G48/5*0.15,0)+IFERROR(H48/5*0.15,0)+IFERROR(I48/5*0.1,0)+IFERROR(J48/5*0.05,0)+IFERROR(K48/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M48" s="77">
+      <c r="M48" s="131">
         <f>IF(L48="","",IF(L48&gt;=0.85,"Meets/Exceeds",IF(L48&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -10907,7 +10917,7 @@
         <f>IF((COUNT(E49)+COUNT(F49)+COUNT(G49)+COUNT(H49)+COUNT(I49)+COUNT(J49)+COUNT(K49))=0,"",IFERROR(E49/5*0.3,0)+IFERROR(F49/5*0.2,0)+IFERROR(G49/5*0.15,0)+IFERROR(H49/5*0.15,0)+IFERROR(I49/5*0.1,0)+IFERROR(J49/5*0.05,0)+IFERROR(K49/5*0.05,0))</f>
         <v/>
       </c>
-      <c r="M49" s="82">
+      <c r="M49" s="132">
         <f>IF(L49="","",IF(L49&gt;=0.85,"Meets/Exceeds",IF(L49&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -11044,7 +11054,7 @@
           <t>Band</t>
         </is>
       </c>
-      <c r="I55" s="116" t="inlineStr">
+      <c r="I55" s="125" t="inlineStr">
         <is>
           <t>Journey notes (where the chain broke / recovered)</t>
         </is>
@@ -11062,7 +11072,7 @@
         </is>
       </c>
       <c r="B56" s="69" t="n"/>
-      <c r="C56" s="77">
+      <c r="C56" s="131">
         <f>COUNT(L5:L17)</f>
         <v/>
       </c>
@@ -11080,7 +11090,7 @@
         <f>IF(D56="","",0.5*D56+0.3*(E56/5)+0.2*(F56/5))</f>
         <v/>
       </c>
-      <c r="H56" s="77">
+      <c r="H56" s="131">
         <f>IF(G56="","",IF(G56&gt;=0.85,"Meets/Exceeds",IF(G56&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -11098,7 +11108,7 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="81" t="inlineStr"/>
       <c r="B57" s="69" t="n"/>
-      <c r="C57" s="77">
+      <c r="C57" s="131">
         <f>IF(A57="","",COUNTIF(B5:B49,A57))</f>
         <v/>
       </c>
@@ -11112,7 +11122,7 @@
         <f>IF(OR(A57="",D57="",E57="",F57=""),"",0.5*D57+0.3*(E57/5)+0.2*(F57/5))</f>
         <v/>
       </c>
-      <c r="H57" s="77">
+      <c r="H57" s="131">
         <f>IF(G57="","",IF(G57&gt;=0.85,"Meets/Exceeds",IF(G57&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -11126,7 +11136,7 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="81" t="inlineStr"/>
       <c r="B58" s="69" t="n"/>
-      <c r="C58" s="82">
+      <c r="C58" s="132">
         <f>IF(A58="","",COUNTIF(B5:B49,A58))</f>
         <v/>
       </c>
@@ -11140,7 +11150,7 @@
         <f>IF(OR(A58="",D58="",E58="",F58=""),"",0.5*D58+0.3*(E58/5)+0.2*(F58/5))</f>
         <v/>
       </c>
-      <c r="H58" s="82">
+      <c r="H58" s="132">
         <f>IF(G58="","",IF(G58&gt;=0.85,"Meets/Exceeds",IF(G58&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -11154,7 +11164,7 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="81" t="inlineStr"/>
       <c r="B59" s="69" t="n"/>
-      <c r="C59" s="77">
+      <c r="C59" s="131">
         <f>IF(A59="","",COUNTIF(B5:B49,A59))</f>
         <v/>
       </c>
@@ -11168,7 +11178,7 @@
         <f>IF(OR(A59="",D59="",E59="",F59=""),"",0.5*D59+0.3*(E59/5)+0.2*(F59/5))</f>
         <v/>
       </c>
-      <c r="H59" s="77">
+      <c r="H59" s="131">
         <f>IF(G59="","",IF(G59&gt;=0.85,"Meets/Exceeds",IF(G59&gt;=0.70,"Developing","Needs Improv.")))</f>
         <v/>
       </c>
@@ -11201,20 +11211,20 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="I55:N55"/>
     <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A57:B57"/>
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A57:B57"/>
     <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A60:N60"/>
-    <mergeCell ref="A54:P54"/>
-    <mergeCell ref="I58:N58"/>
-    <mergeCell ref="I55:N55"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
     <mergeCell ref="I57:N57"/>
+    <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="A2:P2"/>
@@ -11290,7 +11300,7 @@
       <formula>"Maintainer"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="20" operator="equal" dxfId="2">
-      <formula>"Breaker"</formula>
+      <formula>"Regression Contributor"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P49">
@@ -11315,7 +11325,7 @@
       <formula2>5</formula2>
     </dataValidation>
     <dataValidation sqref="O5:O49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Resolver, Progress Builder, Maintainer, Breaker, or N/A." type="list">
-      <formula1>"Resolver,Progress Builder,Maintainer,Breaker,N/A"</formula1>
+      <formula1>"Resolver,Progress Builder,Maintainer,Regression Contributor,N/A"</formula1>
     </dataValidation>
     <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole" operator="between">
       <formula1>0</formula1>

</xml_diff>